<commit_message>
fix: reactor lookup #NAME?/#N/A (MAXIFS->SUMPRODUCT); honest flush_factor default
- D36 latest_date used MAXIFS (Excel 2019+ only -> #NAME? on this build), cascading
  #N/A into flowrate_cal/min_sparge_cal. The LOOKUP(2,1/array) forms also tripped Excel's
  @ implicit-intersection. Rewrote all three as SUMPRODUCT (works in every Excel version,
  no @ pitfalls): latest_date=SUMPRODUCT(MAX(...)), flowrate/min_sparge via masked SUMPRODUCT.
- flush_factor 1.3 -> 1.0 (one headspace flush). The 1.3 had been back-fitted to reproduce
  the 1s schedule; honest computed optimum is 0.78s/3.08min. 1s = 1.28 headspace volumes.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel-modular.xlsx
+++ b/Media/electroPioreactorGasModel-modular.xlsx
@@ -7830,11 +7830,11 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Headspace volumes of CO2 per pulse; &gt;=1 flushes, 1.3 = full sweep + margin.</t>
+          <t>Headspace volumes of CO₂ per pulse. 1.0 = exactly one headspace flush (the minimum that fully sweeps it). Raise for margin.</t>
         </is>
       </c>
     </row>
@@ -7855,7 +7855,7 @@
         </is>
       </c>
       <c r="D36">
-        <f>MAXIFS('CO2 flows'!$O$4:$O$50,'CO2 flows'!$N$4:$N$50,Reactor)</f>
+        <f>SUMPRODUCT(MAX(('CO2 flows'!$N$4:$N$50=Reactor)*'CO2 flows'!$O$4:$O$50))</f>
         <v/>
       </c>
       <c r="E36" t="inlineStr">
@@ -7881,7 +7881,7 @@
         </is>
       </c>
       <c r="D37">
-        <f>LOOKUP(2,1/(('CO2 flows'!$N$4:$N$50=Reactor)*('CO2 flows'!$O$4:$O$50=latest_date)),'CO2 flows'!$P$4:$P$50)</f>
+        <f>SUMPRODUCT(('CO2 flows'!$N$4:$N$50=Reactor)*('CO2 flows'!$O$4:$O$50=latest_date)*'CO2 flows'!$P$4:$P$50)</f>
         <v/>
       </c>
       <c r="E37" t="inlineStr">
@@ -7907,7 +7907,7 @@
         </is>
       </c>
       <c r="D38">
-        <f>LOOKUP(2,1/(('CO2 flows'!$N$4:$N$50=Reactor)*('CO2 flows'!$O$4:$O$50=latest_date)),'CO2 flows'!$Q$4:$Q$50)</f>
+        <f>SUMPRODUCT(('CO2 flows'!$N$4:$N$50=Reactor)*('CO2 flows'!$O$4:$O$50=latest_date)*'CO2 flows'!$Q$4:$Q$50)</f>
         <v/>
       </c>
       <c r="E38" t="inlineStr">

</xml_diff>

<commit_message>
model(modular): add reactor/type/electrode/HOB/media lookup tables + table-driven selector dropdowns
- five vertical lookup tables, natural orientation (entries as rows), stacked top-to-bottom per tab; none side-by-side
- Geometry: reactor->type (22 reactors) and reactor-type geometry+stir-bar (4 types)
- Electrochemistry: electrode table (sparger/porosity/cathode/etaF/z_e_ORR), TBD/gaps pink
- Biology: HOB DO thresholds (min/optimum/impairment/toxic) + media; unknowns marked '?' pink
- Summary: 4 selectors (reactor/electrode/organism/media) with dynamic dropdowns off the vertical key columns
- CO2 flows: moved calibration summary from right-of-raw-data (N-Q) to below it (A49-55); re-pointed Dosing reactor lookup to A51:A80 (SUMPRODUCT)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel-modular.xlsx
+++ b/Media/electroPioreactorGasModel-modular.xlsx
@@ -270,7 +270,7 @@
     <numFmt numFmtId="171" formatCode="0.0000000"/>
     <numFmt numFmtId="172" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -404,6 +404,10 @@
     <font>
       <i val="1"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="17">
@@ -599,7 +603,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -707,6 +711,8 @@
     <xf numFmtId="172" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1057,7 +1063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1454,8 +1460,83 @@
       <c r="C30" s="28" t="n"/>
       <c r="D30" s="29" t="n"/>
     </row>
+    <row r="32">
+      <c r="A32" s="73" t="inlineStr">
+        <is>
+          <t>EXPERIMENT SELECTORS  (dropdowns auto-extend from the lookup tables; wired to calcs next stage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Reactor</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Reactor_sel</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>ed04</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Electrode</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>electrode_sel</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>MMO tube</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>HOB organism</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>organism_sel</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Cupriavidus necator</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>media_sel</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Sydow 2017 minimal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="7">
     <dataValidation sqref="D3" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
       <formula1>"AEP0.1.1,AEP0.2"</formula1>
     </dataValidation>
@@ -1464,6 +1545,18 @@
     </dataValidation>
     <dataValidation sqref="D5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
       <formula1>"0,1,2,3,4,5"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Geometry!$A$53:$A$82</formula1>
+    </dataValidation>
+    <dataValidation sqref="D34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Electrochemistry!$A$32:$A$40</formula1>
+    </dataValidation>
+    <dataValidation sqref="D35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Biology!$A$47:$A$60</formula1>
+    </dataValidation>
+    <dataValidation sqref="D36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Biology!$A$56:$A$64</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1478,7 +1571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:I83"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2652,6 +2745,482 @@
       <c r="E48" t="inlineStr">
         <is>
           <t>From Summary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="73" t="inlineStr">
+        <is>
+          <t>REACTOR LOOKUP  (reactor ID → type)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="69" t="inlineStr">
+        <is>
+          <t>Reactor</t>
+        </is>
+      </c>
+      <c r="B52" s="69" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>imp01</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>AEP0.1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>imp02</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>AEP0.1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>imp03</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>AEP0.1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>imp04</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>AEP0.1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>imp05</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>AEP0.1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>imp06</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>AEP0.1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>ed01</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>AEP0.1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>ed02</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>AEP0.1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>ed03</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>AEP0.1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ed04</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>MEP0.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ed05</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>MEP0.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>ed06</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>AEP0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>ed07</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>AEP0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>ed08</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>AEP0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>imp07</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>AEP0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>imp08</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>AEP0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>imp09</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>AEP0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>imp10</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>AEP0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>imp11</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>AEP0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>imp12</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>AEP0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>nm01</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>AEP0.2a</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>nm02</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>AEP0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="73" t="inlineStr">
+        <is>
+          <t>REACTOR-TYPE LOOKUP  (geometry &amp; stir bar; pulled by type)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="69" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B77" s="69" t="inlineStr">
+        <is>
+          <t>Pioreactor</t>
+        </is>
+      </c>
+      <c r="C77" s="69" t="inlineStr">
+        <is>
+          <t>vial (mL)</t>
+        </is>
+      </c>
+      <c r="D77" s="69" t="inlineStr">
+        <is>
+          <t>usable depth (mm)</t>
+        </is>
+      </c>
+      <c r="E77" s="69" t="inlineStr">
+        <is>
+          <t>max working (mL)</t>
+        </is>
+      </c>
+      <c r="F77" s="69" t="inlineStr">
+        <is>
+          <t>total vial (mL)</t>
+        </is>
+      </c>
+      <c r="G77" s="69" t="inlineStr">
+        <is>
+          <t>vial OD (mm)</t>
+        </is>
+      </c>
+      <c r="H77" s="69" t="inlineStr">
+        <is>
+          <t>stir bar L (mm)</t>
+        </is>
+      </c>
+      <c r="I77" s="69" t="inlineStr">
+        <is>
+          <t>stir bar dia (mm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>AEP0.1.1</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>20</v>
+      </c>
+      <c r="D78" t="n">
+        <v>55</v>
+      </c>
+      <c r="E78" t="n">
+        <v>16</v>
+      </c>
+      <c r="F78" t="n">
+        <v>20</v>
+      </c>
+      <c r="G78" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="H78" t="n">
+        <v>12</v>
+      </c>
+      <c r="I78" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>MEP0.3</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>20</v>
+      </c>
+      <c r="D79" t="n">
+        <v>55</v>
+      </c>
+      <c r="E79" t="n">
+        <v>16</v>
+      </c>
+      <c r="F79" t="n">
+        <v>20</v>
+      </c>
+      <c r="G79" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="H79" t="n">
+        <v>12</v>
+      </c>
+      <c r="I79" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>AEP0.2</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>40</v>
+      </c>
+      <c r="D80" t="n">
+        <v>95</v>
+      </c>
+      <c r="E80" t="n">
+        <v>30</v>
+      </c>
+      <c r="F80" t="n">
+        <v>42</v>
+      </c>
+      <c r="G80" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="H80" t="n">
+        <v>15</v>
+      </c>
+      <c r="I80" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>AEP0.2a</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>40</v>
+      </c>
+      <c r="D81" t="n">
+        <v>95</v>
+      </c>
+      <c r="E81" t="n">
+        <v>30</v>
+      </c>
+      <c r="F81" t="n">
+        <v>42</v>
+      </c>
+      <c r="G81" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="H81" t="n">
+        <v>15</v>
+      </c>
+      <c r="I81" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="72" t="inlineStr">
+        <is>
+          <t>40 mL OD = 20 mL diameter (Pioreactor source); depths/volumes confirm by measurement.</t>
         </is>
       </c>
     </row>
@@ -2667,7 +3236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3300,6 +3869,190 @@
       <c r="E27" t="inlineStr">
         <is>
           <t>From Dosing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="73" t="inlineStr">
+        <is>
+          <t>ELECTRODE LOOKUP  (selecting the electrode sets sparger, porosity, cathode)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="69" t="inlineStr">
+        <is>
+          <t>Electrode</t>
+        </is>
+      </c>
+      <c r="B31" s="69" t="inlineStr">
+        <is>
+          <t>anode material</t>
+        </is>
+      </c>
+      <c r="C31" s="69" t="inlineStr">
+        <is>
+          <t>anode dia (mm)</t>
+        </is>
+      </c>
+      <c r="D31" s="69" t="inlineStr">
+        <is>
+          <t>sparger</t>
+        </is>
+      </c>
+      <c r="E31" s="69" t="inlineStr">
+        <is>
+          <t>sinter porosity</t>
+        </is>
+      </c>
+      <c r="F31" s="69" t="inlineStr">
+        <is>
+          <t>cathode</t>
+        </is>
+      </c>
+      <c r="G31" s="69" t="inlineStr">
+        <is>
+          <t>cathode dia (mm)</t>
+        </is>
+      </c>
+      <c r="H31" s="69" t="inlineStr">
+        <is>
+          <t>etaF</t>
+        </is>
+      </c>
+      <c r="I31" s="69" t="inlineStr">
+        <is>
+          <t>z_e_ORR</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Pt/Ti rod</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Pt/Ti</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>6</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Tube</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>SS rod</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>6</v>
+      </c>
+      <c r="H32" s="74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>MMO rod</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>MMO</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>6</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Tube</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>SS rod</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>6</v>
+      </c>
+      <c r="H33" s="74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>MMO tube</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>MMO</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>6</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Sintered</t>
+        </is>
+      </c>
+      <c r="E34" s="74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>SS rod</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>6</v>
+      </c>
+      <c r="H34" s="74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="72" t="inlineStr">
+        <is>
+          <t>z_e_ORR=2 assumed (peroxide, non-Pt SS cathode, neutral pH); etaF unmeasured - both live here per electrode.</t>
         </is>
       </c>
     </row>
@@ -3323,7 +4076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4341,6 +5094,290 @@
       <c r="E42" t="inlineStr">
         <is>
           <t>From Geometry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="73" t="inlineStr">
+        <is>
+          <t>HOB LOOKUP  (dissolved O₂ thresholds, mg/L)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="69" t="inlineStr">
+        <is>
+          <t>Organism</t>
+        </is>
+      </c>
+      <c r="B46" s="69" t="inlineStr">
+        <is>
+          <t>minimum DO</t>
+        </is>
+      </c>
+      <c r="C46" s="69" t="inlineStr">
+        <is>
+          <t>optimum DO</t>
+        </is>
+      </c>
+      <c r="D46" s="69" t="inlineStr">
+        <is>
+          <t>impairment DO</t>
+        </is>
+      </c>
+      <c r="E46" s="69" t="inlineStr">
+        <is>
+          <t>toxic DO</t>
+        </is>
+      </c>
+      <c r="F46" s="69" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Cupriavidus necator</t>
+        </is>
+      </c>
+      <c r="B47" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="D47" t="n">
+        <v>3</v>
+      </c>
+      <c r="E47" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Amer &amp; Kim 2023; Wilde &amp; Schlegel 1982</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Xanthobacter autotrophicus</t>
+        </is>
+      </c>
+      <c r="B48" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="C48" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D48" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Wilde &amp; Schlegel 1982 (~0.30 atm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Xanthobacter flavus</t>
+        </is>
+      </c>
+      <c r="B49" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="C49" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D49" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E49" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>no species data — assume genus ~11.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Xanthobacter tagetidis</t>
+        </is>
+      </c>
+      <c r="B50" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="C50" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D50" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E50" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>no species data — assume genus ~11.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Cupriavidus metallidurans</t>
+        </is>
+      </c>
+      <c r="B51" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="C51" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D51" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E51" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>no species data — assume genus ~11.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>UdG (mixed)</t>
+        </is>
+      </c>
+      <c r="B52" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="C52" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D52" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E52" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Rovira-Alsina 2025; Pous 2022/23</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="73" t="inlineStr">
+        <is>
+          <t>MEDIA LOOKUP</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="69" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="B55" s="69" t="inlineStr">
+        <is>
+          <t>buffer</t>
+        </is>
+      </c>
+      <c r="C55" s="69" t="inlineStr">
+        <is>
+          <t>buffer conc (mM)</t>
+        </is>
+      </c>
+      <c r="D55" s="69" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="E55" s="69" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Sydow 2017 minimal</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>phosphate</t>
+        </is>
+      </c>
+      <c r="C56" s="74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>low-chloride, organic-free</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Sydow et al. 2017</t>
         </is>
       </c>
     </row>
@@ -7855,7 +8892,7 @@
         </is>
       </c>
       <c r="D36">
-        <f>SUMPRODUCT(MAX(('CO2 flows'!$N$4:$N$50=Reactor)*'CO2 flows'!$O$4:$O$50))</f>
+        <f>SUMPRODUCT(MAX(('CO2 flows'!$A$51:$A$80=Reactor)*'CO2 flows'!$B$51:$B$80))</f>
         <v/>
       </c>
       <c r="E36" t="inlineStr">
@@ -7881,7 +8918,7 @@
         </is>
       </c>
       <c r="D37">
-        <f>SUMPRODUCT(('CO2 flows'!$N$4:$N$50=Reactor)*('CO2 flows'!$O$4:$O$50=latest_date)*'CO2 flows'!$P$4:$P$50)</f>
+        <f>SUMPRODUCT(('CO2 flows'!$A$51:$A$80=Reactor)*('CO2 flows'!$B$51:$B$80=latest_date)*'CO2 flows'!$C$51:$C$80)</f>
         <v/>
       </c>
       <c r="E37" t="inlineStr">
@@ -7907,7 +8944,7 @@
         </is>
       </c>
       <c r="D38">
-        <f>SUMPRODUCT(('CO2 flows'!$N$4:$N$50=Reactor)*('CO2 flows'!$O$4:$O$50=latest_date)*'CO2 flows'!$Q$4:$Q$50)</f>
+        <f>SUMPRODUCT(('CO2 flows'!$A$51:$A$80=Reactor)*('CO2 flows'!$B$51:$B$80=latest_date)*'CO2 flows'!$D$51:$D$80)</f>
         <v/>
       </c>
       <c r="E38" t="inlineStr">
@@ -7954,7 +8991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q47"/>
+  <dimension ref="A1:S55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="9"/>
@@ -8019,11 +9056,7 @@
           <t>KEY</t>
         </is>
       </c>
-      <c r="N2" s="69" t="inlineStr">
-        <is>
-          <t>CALIBRATION SUMMARY (model lookup source)</t>
-        </is>
-      </c>
+      <c r="N2" s="69" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="58" t="n"/>
@@ -8068,26 +9101,10 @@
           <t>Flowrate set by inspection, as maximum to not give bubbles rising into vial neck</t>
         </is>
       </c>
-      <c r="N3" s="69" t="inlineStr">
-        <is>
-          <t>Reactor</t>
-        </is>
-      </c>
-      <c r="O3" s="69" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="P3" s="69" t="inlineStr">
-        <is>
-          <t>Flowrate</t>
-        </is>
-      </c>
-      <c r="Q3" s="69" t="inlineStr">
-        <is>
-          <t>Min sparge</t>
-        </is>
-      </c>
+      <c r="N3" s="69" t="n"/>
+      <c r="O3" s="69" t="n"/>
+      <c r="P3" s="69" t="n"/>
+      <c r="Q3" s="69" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8109,20 +9126,8 @@
           <t>First or last data point removed as suspect outlier</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>ed04</t>
-        </is>
-      </c>
-      <c r="O4" s="70" t="n">
-        <v>46190</v>
-      </c>
-      <c r="P4" s="71" t="n">
-        <v>3.33</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.25</v>
-      </c>
+      <c r="O4" s="70" t="n"/>
+      <c r="P4" s="71" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8154,11 +9159,7 @@
         <f>AVERAGE(G5)</f>
         <v/>
       </c>
-      <c r="N5" s="72" t="inlineStr">
-        <is>
-          <t>(add a row per reactor/date as calibrations are collected)</t>
-        </is>
-      </c>
+      <c r="N5" s="72" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8226,11 +9227,7 @@
           <t>CO2 collected in measuring cyclinder over CO2-saturated water</t>
         </is>
       </c>
-      <c r="N7" s="69" t="inlineStr">
-        <is>
-          <t>Min sparge justification:</t>
-        </is>
-      </c>
+      <c r="N7" s="69" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8266,11 +9263,6 @@
           <t>Collected using inlet CO2 tube rather than outlet as MEP vialcap leaking</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>0.25 s. Deliveries are exactly repeatable at 0.25 s (1 ml every shot) and at 0.5 s (2 ml). At 0.2 s and below the per-pulse flowrate is erratic (2-6 ml/s): the ~0.4 ml fixed open/close bolus and millisecond timing jitter dominate, so dosing stops being linear or repeatable. Flowrate 3.33 ml/s = inspection-set max (no bubbles into the vial neck), confirmed by the long-pulse calibration slope.</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -9281,6 +10273,72 @@
     </row>
     <row r="47">
       <c r="B47" s="66" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="73" t="inlineStr">
+        <is>
+          <t>CALIBRATION SUMMARY (model lookup source — latest date per reactor is used)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="69" t="inlineStr">
+        <is>
+          <t>Reactor</t>
+        </is>
+      </c>
+      <c r="B50" s="69" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C50" s="69" t="inlineStr">
+        <is>
+          <t>Flowrate (ml/s)</t>
+        </is>
+      </c>
+      <c r="D50" s="69" t="inlineStr">
+        <is>
+          <t>Min sparge (s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ed04</t>
+        </is>
+      </c>
+      <c r="B51" s="70" t="n">
+        <v>46190</v>
+      </c>
+      <c r="C51" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="72" t="inlineStr">
+        <is>
+          <t>(add a row per reactor/date as calibrations are collected)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="73" t="inlineStr">
+        <is>
+          <t>Min sparge justification</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>0.25 s. Repeatable at 0.25 s (1 ml/shot) and 0.5 s (2 ml); at &lt;=0.2 s the per-pulse flowrate is erratic (2-6 ml/s) - the ~0.4 ml fixed open/close bolus and timing jitter dominate. Flowrate 3.33 ml/s = inspection-set max (no bubbles into the neck), confirmed by the long-pulse slope.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="H5:H46">

</xml_diff>

<commit_message>
model(modular): wire electrode + organism-DO selectors; add steady-state DO band check (Stage 2b)
- Electrochemistry: electrode_sel -> sparger (repointed Mass Transfer to it) and z_e_ORR via electrode table; Summary sparger dropdown retired (now shows electrode-resolved value)
- Biology: organism_sel -> minimum/optimum/impairment/toxic DO (ISNUMBER-guarded; gaps return NA, minimum DO flagged pink)
- Mass Transfer: target DO fraction now organism-driven (optimum/inhibition = 0.226 for C. necator, was an arbitrary 0.5)
- Mass Transfer: steady-state DO under surface stripping (DO_ss) + band checks vs organism optimum/minimum; at central kL_surf DO_ss~1.9 mg/L (surface sufficient), result dominated by kL_surf uncertainty
- Summary: surfaces DO_ss and the two band checks

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel-modular.xlsx
+++ b/Media/electroPioreactorGasModel-modular.xlsx
@@ -87,6 +87,8 @@
     <definedName name="z_e_H2" localSheetId="2">Electrochemistry!$D$9</definedName>
     <definedName name="z_e_O2" localSheetId="2">Electrochemistry!$D$10</definedName>
     <definedName name="z_e_ORR" localSheetId="2">Electrochemistry!$D$20</definedName>
+    <definedName name="electrode_sel" localSheetId="2">Electrochemistry!$D$38</definedName>
+    <definedName name="sparger_e" localSheetId="2">Electrochemistry!$D$39</definedName>
     <definedName name="bio_CO2" localSheetId="3">Biology!$D$5</definedName>
     <definedName name="bio_H2" localSheetId="3">Biology!$D$3</definedName>
     <definedName name="bio_O2" localSheetId="3">Biology!$D$4</definedName>
@@ -125,6 +127,11 @@
     <definedName name="T_K" localSheetId="3">Biology!$D$11</definedName>
     <definedName name="T_ref" localSheetId="3">Biology!$D$16</definedName>
     <definedName name="V_charge" localSheetId="3">Biology!$D$42</definedName>
+    <definedName name="organism_sel" localSheetId="3">Biology!$D$57</definedName>
+    <definedName name="DO_min" localSheetId="3">Biology!$D$58</definedName>
+    <definedName name="DO_opt" localSheetId="3">Biology!$D$59</definedName>
+    <definedName name="DO_impair" localSheetId="3">Biology!$D$60</definedName>
+    <definedName name="DO_toxic" localSheetId="3">Biology!$D$61</definedName>
     <definedName name="a_int" localSheetId="4">'Mass Transfer'!$D$25</definedName>
     <definedName name="a_surf" localSheetId="4">'Mass Transfer'!$D$48</definedName>
     <definedName name="A_x" localSheetId="4">'Mass Transfer'!$D$96</definedName>
@@ -222,6 +229,13 @@
     <definedName name="We_orifice" localSheetId="4">'Mass Transfer'!$D$39</definedName>
     <definedName name="y_O2_vent" localSheetId="4">'Mass Transfer'!$D$52</definedName>
     <definedName name="flush_factor" localSheetId="4">'Mass Transfer'!$D$102</definedName>
+    <definedName name="DO_opt" localSheetId="4">'Mass Transfer'!$D$103</definedName>
+    <definedName name="DO_impair" localSheetId="4">'Mass Transfer'!$D$104</definedName>
+    <definedName name="DO_toxic" localSheetId="4">'Mass Transfer'!$D$105</definedName>
+    <definedName name="DO_min" localSheetId="4">'Mass Transfer'!$D$106</definedName>
+    <definedName name="DO_ss" localSheetId="4">'Mass Transfer'!$D$109</definedName>
+    <definedName name="DO_ss_vs_opt" localSheetId="4">'Mass Transfer'!$D$110</definedName>
+    <definedName name="DO_ss_vs_min" localSheetId="4">'Mass Transfer'!$D$111</definedName>
     <definedName name="CO2_cons" localSheetId="5">Dosing!$D$25</definedName>
     <definedName name="CO2_pulse" localSheetId="5">Dosing!$D$10</definedName>
     <definedName name="CO2_sd_ratio" localSheetId="5">Dosing!$D$14</definedName>
@@ -509,7 +523,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -649,11 +663,53 @@
         <color theme="9"/>
       </bottom>
     </border>
+    <border>
+      <left style="medium">
+        <color theme="8"/>
+      </left>
+      <right style="medium">
+        <color theme="8"/>
+      </right>
+      <top style="medium">
+        <color theme="8"/>
+      </top>
+      <bottom style="medium">
+        <color theme="8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="5"/>
+      </left>
+      <right style="medium">
+        <color theme="5"/>
+      </right>
+      <top style="medium">
+        <color theme="5"/>
+      </top>
+      <bottom style="medium">
+        <color theme="5"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="6"/>
+      </left>
+      <right style="medium">
+        <color theme="6"/>
+      </right>
+      <top style="medium">
+        <color theme="6"/>
+      </top>
+      <bottom style="medium">
+        <color theme="6"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -770,6 +826,11 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="23" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1120,7 +1181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1192,7 +1253,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Sparger type</t>
+          <t>Sparger type (resolved from electrode)</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -1205,10 +1266,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D4" s="30" t="inlineStr">
-        <is>
-          <t>Sintered</t>
-        </is>
+      <c r="D4" s="82">
+        <f>Electrochemistry!$D$39</f>
+        <v/>
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
@@ -1602,11 +1662,41 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Steady-state DO (surface, mg/L)</t>
+        </is>
+      </c>
+      <c r="D39" s="83">
+        <f>'Mass Transfer'!$D$109</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>DO vs organism optimum</t>
+        </is>
+      </c>
+      <c r="D40" s="83">
+        <f>'Mass Transfer'!$D$110</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>DO vs organism minimum</t>
+        </is>
+      </c>
+      <c r="D41" s="83">
+        <f>'Mass Transfer'!$D$111</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation sqref="D4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
-      <formula1>"Tube,Sintered"</formula1>
-    </dataValidation>
+  <dataValidations count="5">
     <dataValidation sqref="D5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
       <formula1>"0,1,2,3,4,5"</formula1>
     </dataValidation>
@@ -3332,7 +3422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3822,8 +3912,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D20" s="24" t="n">
-        <v>4</v>
+      <c r="D20" s="77">
+        <f>VLOOKUP(electrode_sel,$A$32:$I$34,9,FALSE)</f>
+        <v/>
       </c>
       <c r="E20" s="25" t="inlineStr">
         <is>
@@ -4150,6 +4241,38 @@
         <is>
           <t>z_e_ORR=2 assumed (peroxide, non-Pt SS cathode, neutral pH); etaF unmeasured - both live here per electrode.</t>
         </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>(import) Electrode selection</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>electrode_sel</t>
+        </is>
+      </c>
+      <c r="D38" s="79">
+        <f>Summary!$D$34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Sparger (from electrode)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>sparger_e</t>
+        </is>
+      </c>
+      <c r="D39" s="80">
+        <f>VLOOKUP(electrode_sel,$A$32:$I$34,4,FALSE)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -4172,7 +4295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5475,6 +5598,86 @@
         <is>
           <t>Sydow et al. 2017</t>
         </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>(import) HOB organism</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>organism_sel</t>
+        </is>
+      </c>
+      <c r="D57" s="79">
+        <f>Summary!$D$35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Minimum DO (organism)</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>DO_min</t>
+        </is>
+      </c>
+      <c r="D58" s="84">
+        <f>IF(ISNUMBER(VLOOKUP(organism_sel,$A$47:$F$52,2,FALSE)),VLOOKUP(organism_sel,$A$47:$F$52,2,FALSE),NA())</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Optimum DO (organism)</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>DO_opt</t>
+        </is>
+      </c>
+      <c r="D59" s="80">
+        <f>IF(ISNUMBER(VLOOKUP(organism_sel,$A$47:$F$52,3,FALSE)),VLOOKUP(organism_sel,$A$47:$F$52,3,FALSE),NA())</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Impairment DO (organism)</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>DO_impair</t>
+        </is>
+      </c>
+      <c r="D60" s="80">
+        <f>IF(ISNUMBER(VLOOKUP(organism_sel,$A$47:$F$52,4,FALSE)),VLOOKUP(organism_sel,$A$47:$F$52,4,FALSE),NA())</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Toxic/inhibition DO (organism)</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>DO_toxic</t>
+        </is>
+      </c>
+      <c r="D61" s="80">
+        <f>IF(ISNUMBER(VLOOKUP(organism_sel,$A$47:$F$52,5,FALSE)),VLOOKUP(organism_sel,$A$47:$F$52,5,FALSE),NA())</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -5506,7 +5709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E102"/>
+  <dimension ref="A1:E111"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7042,7 +7245,7 @@
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>Target dissolved-O₂ ceiling fraction</t>
+          <t>Target DO fraction (organism optimum / inhibition)</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
@@ -7055,8 +7258,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D61" s="52" t="n">
-        <v>0.5</v>
+      <c r="D61" s="85">
+        <f>IF(AND(ISNUMBER(DO_opt),ISNUMBER(DO_toxic)),DO_opt/DO_toxic,0.5)</f>
+        <v/>
       </c>
       <c r="E61" s="25" t="inlineStr">
         <is>
@@ -8008,7 +8212,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>(import) Sparger type</t>
+          <t>(import) Sparger type (from electrode)</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -8021,8 +8225,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D100">
-        <f>Summary!$D$4</f>
+      <c r="D100" s="82">
+        <f>Electrochemistry!$D$39</f>
         <v/>
       </c>
       <c r="E100" t="inlineStr">
@@ -8055,6 +8259,125 @@
         <is>
           <t>From Dosing.</t>
         </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>(import) Optimum DO (organism)</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>DO_opt</t>
+        </is>
+      </c>
+      <c r="D103" s="86">
+        <f>Biology!$D$59</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>(import) Impairment DO (organism)</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>DO_impair</t>
+        </is>
+      </c>
+      <c r="D104" s="86">
+        <f>Biology!$D$60</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>(import) Toxic/inhibition DO (organism)</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>DO_toxic</t>
+        </is>
+      </c>
+      <c r="D105" s="86">
+        <f>Biology!$D$61</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>(import) Minimum DO (organism)</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>DO_min</t>
+        </is>
+      </c>
+      <c r="D106" s="86">
+        <f>Biology!$D$58</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="69" t="inlineStr">
+        <is>
+          <t>STEADY-STATE DO CHECK (surface stripping vs organism band)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Steady-state DO under surface stripping</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>DO_ss</t>
+        </is>
+      </c>
+      <c r="D109" s="80">
+        <f>O2_excess/(kLa_surf_used*3600*(V_charge/1000000))*32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  DO_ss vs optimum (organism)</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>DO_ss_vs_opt</t>
+        </is>
+      </c>
+      <c r="D110" s="80">
+        <f>IF(ISNUMBER(DO_opt),IF(DO_ss&lt;=DO_opt,"at/under optimum",IF(DO_ss&lt;DO_impair,"above optimum, under impairment","OVER IMPAIRMENT - surface strip insufficient")),"organism optimum unknown")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  DO_ss vs minimum (organism)</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>DO_ss_vs_min</t>
+        </is>
+      </c>
+      <c r="D111" s="80">
+        <f>IF(ISNUMBER(DO_min),IF(DO_ss&gt;=DO_min,"above minimum","BELOW MINIMUM"),"minimum DO unknown - measure")</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
model(modular): CO2 flows back to one table; lookup reads nominal flowrate + min sparge
- removed the wrongly-added second calibration table (rows 49-76)
- single raw table gains one column: nominal flowrate (J); minimum sparge already existed (col I)
- ed04 calibration entered inline (nominal 3.33 ml/s, min sparge 0.25 s); researchers add a row the same way
- Dosing lookup re-pointed at the single table A4:J200, keyed reactor + latest calibrated date, no type column; warns when a reactor has no calibration row

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel-modular.xlsx
+++ b/Media/electroPioreactorGasModel-modular.xlsx
@@ -268,9 +268,8 @@
     <definedName name="latest_date" localSheetId="5">Dosing!$D$36</definedName>
     <definedName name="flowrate_cal" localSheetId="5">Dosing!$D$37</definedName>
     <definedName name="min_sparge_cal" localSheetId="5">Dosing!$D$38</definedName>
-    <definedName name="cal_exact_n" localSheetId="5">Dosing!$D$39</definedName>
-    <definedName name="cal_type" localSheetId="5">Dosing!$D$40</definedName>
     <definedName name="cal_warning" localSheetId="5">Dosing!$D$41</definedName>
+    <definedName name="has_cal" localSheetId="5">Dosing!$D$39</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
@@ -9311,7 +9310,7 @@
         </is>
       </c>
       <c r="D36" s="80">
-        <f>IF(cal_exact_n&gt;0,SUMPRODUCT(MAX(('CO2 flows'!$A$51:$A$70=Reactor)*'CO2 flows'!$B$51:$B$70)),SUMPRODUCT(MAX(('CO2 flows'!$E$51:$E$70=cal_type)*'CO2 flows'!$B$51:$B$70)))</f>
+        <f>SUMPRODUCT(MAX(('CO2 flows'!$A$4:$A$200=Reactor)*('CO2 flows'!$J$4:$J$200&gt;0)*'CO2 flows'!$B$4:$B$200))</f>
         <v/>
       </c>
       <c r="E36" t="inlineStr">
@@ -9337,7 +9336,7 @@
         </is>
       </c>
       <c r="D37" s="80">
-        <f>IF(cal_exact_n&gt;0,SUMPRODUCT(('CO2 flows'!$A$51:$A$70=Reactor)*('CO2 flows'!$B$51:$B$70=latest_date)*'CO2 flows'!$C$51:$C$70)/MAX(1,SUMPRODUCT(('CO2 flows'!$A$51:$A$70=Reactor)*('CO2 flows'!$B$51:$B$70=latest_date)*1)),SUMPRODUCT(('CO2 flows'!$E$51:$E$70=cal_type)*('CO2 flows'!$B$51:$B$70=latest_date)*'CO2 flows'!$C$51:$C$70)/MAX(1,SUMPRODUCT(('CO2 flows'!$E$51:$E$70=cal_type)*('CO2 flows'!$B$51:$B$70=latest_date)*1)))</f>
+        <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$200=Reactor)*('CO2 flows'!$B$4:$B$200=latest_date)*'CO2 flows'!$J$4:$J$200)/MAX(1,SUMPRODUCT(('CO2 flows'!$A$4:$A$200=Reactor)*('CO2 flows'!$B$4:$B$200=latest_date)*('CO2 flows'!$J$4:$J$200&gt;0)*1))</f>
         <v/>
       </c>
       <c r="E37" t="inlineStr">
@@ -9363,7 +9362,7 @@
         </is>
       </c>
       <c r="D38" s="80">
-        <f>IF(cal_exact_n&gt;0,SUMPRODUCT(('CO2 flows'!$A$51:$A$70=Reactor)*('CO2 flows'!$B$51:$B$70=latest_date)*'CO2 flows'!$D$51:$D$70)/MAX(1,SUMPRODUCT(('CO2 flows'!$A$51:$A$70=Reactor)*('CO2 flows'!$B$51:$B$70=latest_date)*1)),SUMPRODUCT(('CO2 flows'!$E$51:$E$70=cal_type)*('CO2 flows'!$B$51:$B$70=latest_date)*'CO2 flows'!$D$51:$D$70)/MAX(1,SUMPRODUCT(('CO2 flows'!$E$51:$E$70=cal_type)*('CO2 flows'!$B$51:$B$70=latest_date)*1)))</f>
+        <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$200=Reactor)*('CO2 flows'!$B$4:$B$200=latest_date)*'CO2 flows'!$I$4:$I$200)/MAX(1,SUMPRODUCT(('CO2 flows'!$A$4:$A$200=Reactor)*('CO2 flows'!$B$4:$B$200=latest_date)*('CO2 flows'!$J$4:$J$200&gt;0)*1))</f>
         <v/>
       </c>
       <c r="E38" t="inlineStr">
@@ -9375,34 +9374,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>calibration rows for this reactor</t>
+          <t>reactor has a calibration row?</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>cal_exact_n</t>
+          <t>has_cal</t>
         </is>
       </c>
       <c r="D39" s="80">
-        <f>SUMPRODUCT(('CO2 flows'!$A$51:$A$70=Reactor)*1)</f>
+        <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$200=Reactor)*('CO2 flows'!$J$4:$J$200&gt;0)*1)</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>reactor type (for nearest-match)</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>cal_type</t>
-        </is>
-      </c>
-      <c r="D40" s="80">
-        <f>IFERROR(VLOOKUP(Reactor,Geometry!$A$53:$B$74,2,FALSE),"?")</f>
-        <v/>
-      </c>
+      <c r="D40" s="80" t="n"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -9416,7 +9402,7 @@
         </is>
       </c>
       <c r="D41" s="80">
-        <f>IF(cal_exact_n&gt;0,"exact: "&amp;Reactor,"NEAREST TYPE ("&amp;cal_type&amp;") - no calibration for "&amp;Reactor)</f>
+        <f>IF(has_cal&gt;0,"calibrated: "&amp;Reactor,"NO CALIBRATION for "&amp;Reactor&amp;" - add a row in CO2 flows with nominal flowrate + minimum sparge")</f>
         <v/>
       </c>
     </row>
@@ -9518,6 +9504,11 @@
           <t>minimum sparge</t>
         </is>
       </c>
+      <c r="J2" s="69" t="inlineStr">
+        <is>
+          <t>nominal flowrate</t>
+        </is>
+      </c>
       <c r="L2" s="59" t="inlineStr">
         <is>
           <t>KEY</t>
@@ -9563,6 +9554,11 @@
           <t>s</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>ml/s</t>
+        </is>
+      </c>
       <c r="L3" s="68" t="inlineStr">
         <is>
           <t>Flowrate set by inspection, as maximum to not give bubbles rising into vial neck</t>
@@ -9588,6 +9584,12 @@
       <c r="D4" t="n">
         <v>0</v>
       </c>
+      <c r="I4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J4" t="n">
+        <v>3.33</v>
+      </c>
       <c r="L4" s="67" t="inlineStr">
         <is>
           <t>First or last data point removed as suspect outlier</t>
@@ -10741,204 +10743,55 @@
     <row r="47">
       <c r="B47" s="66" t="n"/>
     </row>
+    <row r="48"/>
     <row r="49">
-      <c r="A49" s="73" t="inlineStr">
-        <is>
-          <t>CALIBRATION SUMMARY (model lookup source — latest date per reactor is used)</t>
-        </is>
-      </c>
+      <c r="A49" s="73" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="69" t="inlineStr">
-        <is>
-          <t>Reactor</t>
-        </is>
-      </c>
-      <c r="B50" s="69" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C50" s="69" t="inlineStr">
-        <is>
-          <t>Flowrate (ml/s)</t>
-        </is>
-      </c>
-      <c r="D50" s="69" t="inlineStr">
-        <is>
-          <t>Min sparge (s)</t>
-        </is>
-      </c>
-      <c r="E50" s="69" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
+      <c r="A50" s="69" t="n"/>
+      <c r="B50" s="69" t="n"/>
+      <c r="C50" s="69" t="n"/>
+      <c r="D50" s="69" t="n"/>
+      <c r="E50" s="69" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>ed04</t>
-        </is>
-      </c>
-      <c r="B51" s="70" t="n">
-        <v>46190</v>
-      </c>
-      <c r="C51" t="n">
-        <v>3.33</v>
-      </c>
-      <c r="D51" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E51">
-        <f>IFERROR(VLOOKUP(A51,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
+      <c r="B51" s="70" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="72" t="n"/>
-      <c r="E52">
-        <f>IFERROR(VLOOKUP(A52,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="E53">
-        <f>IFERROR(VLOOKUP(A53,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
-    </row>
+    </row>
+    <row r="53"/>
     <row r="54">
       <c r="A54" s="73" t="n"/>
-      <c r="E54">
-        <f>IFERROR(VLOOKUP(A54,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="E55">
-        <f>IFERROR(VLOOKUP(A55,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="E56">
-        <f>IFERROR(VLOOKUP(A56,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="E57">
-        <f>IFERROR(VLOOKUP(A57,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="E58">
-        <f>IFERROR(VLOOKUP(A58,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59">
-      <c r="E59">
-        <f>IFERROR(VLOOKUP(A59,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="E60">
-        <f>IFERROR(VLOOKUP(A60,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="E61">
-        <f>IFERROR(VLOOKUP(A61,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="E62">
-        <f>IFERROR(VLOOKUP(A62,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="E63">
-        <f>IFERROR(VLOOKUP(A63,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="E64">
-        <f>IFERROR(VLOOKUP(A64,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65">
-      <c r="E65">
-        <f>IFERROR(VLOOKUP(A65,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66">
-      <c r="E66">
-        <f>IFERROR(VLOOKUP(A66,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67">
-      <c r="E67">
-        <f>IFERROR(VLOOKUP(A67,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68">
-      <c r="E68">
-        <f>IFERROR(VLOOKUP(A68,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69">
-      <c r="E69">
-        <f>IFERROR(VLOOKUP(A69,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70">
-      <c r="E70">
-        <f>IFERROR(VLOOKUP(A70,Geometry!$A$53:$B$74,2,FALSE),"")</f>
-        <v/>
-      </c>
-    </row>
+    </row>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
     <row r="72">
-      <c r="A72" s="72" t="inlineStr">
-        <is>
-          <t>Add one row per reactor + calibration date below the header (row 50); rows 51-70 are the lookup range.</t>
-        </is>
-      </c>
+      <c r="A72" s="72" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="72" t="inlineStr">
-        <is>
-          <t>The latest date for a reactor is used; if a reactor has no row, the latest row of the same reactor type is used (flagged).</t>
-        </is>
-      </c>
-    </row>
+      <c r="A73" s="72" t="n"/>
+    </row>
+    <row r="74"/>
     <row r="75">
-      <c r="A75" s="73" t="inlineStr">
-        <is>
-          <t>Min sparge justification</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>0.25 s. Repeatable at 0.25 s (1 ml/shot) and 0.5 s (2 ml); at &lt;=0.2 s the per-pulse flowrate is erratic (2-6 ml/s) - the ~0.4 ml fixed open/close bolus and timing jitter dominate. Flowrate 3.33 ml/s = inspection-set max (no bubbles into the neck), confirmed by the long-pulse slope.</t>
-        </is>
-      </c>
-    </row>
+      <c r="A75" s="73" t="n"/>
+    </row>
+    <row r="76"/>
   </sheetData>
   <conditionalFormatting sqref="H5:H46">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
model(modular): consolidate all experiment inputs on front page + warnings, improvements, CF, hyperlinks (Stage 3)
- Summary now holds every experiment-to-experiment input: reactor/electrode/organism/media selectors plus LED intensity, stirrer rpm, media volume, temperature, ambient pressure; the specialist tabs import these (control surface inverted)
- Media volume input overrides V_charge when set; warns if it exceeds max working volume or the liquid level exceeds usable depth
- Tip-speed shear flag at >1.5 m/s with citation (BioProcess International cell-culture norm; precautionary for robust HOB)
- Ranked improvements table (impact x effort): kL_surf, etaF, organism min DO, per-reactor flow calibration, uptake ratio, sinter porosity, ambient pressure
- 'From <tab>' hyperlinks on Summary result rows jump to the source cell; traffic-light conditional formatting on output flags; black borders on every Summary-referencing cell

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel-modular.xlsx
+++ b/Media/electroPioreactorGasModel-modular.xlsx
@@ -18,6 +18,11 @@
     <definedName name="por_grade" localSheetId="0">Summary!$D$5</definedName>
     <definedName name="rx_ver" localSheetId="0">Summary!$D$3</definedName>
     <definedName name="sparger" localSheetId="0">Summary!$D$4</definedName>
+    <definedName name="led_intensity" localSheetId="0">Summary!$D$37</definedName>
+    <definedName name="stir_rpm_set" localSheetId="0">Summary!$D$38</definedName>
+    <definedName name="media_volume" localSheetId="0">Summary!$D$39</definedName>
+    <definedName name="temp_C" localSheetId="0">Summary!$D$40</definedName>
+    <definedName name="P_atm_set" localSheetId="0">Summary!$D$41</definedName>
     <definedName name="A_x" localSheetId="1">Geometry!$D$16</definedName>
     <definedName name="D_int" localSheetId="1">Geometry!$D$17</definedName>
     <definedName name="D_int_1" localSheetId="1">Geometry!$D$7</definedName>
@@ -64,6 +69,9 @@
     <definedName name="reactor_sel" localSheetId="1">Geometry!$D$48</definedName>
     <definedName name="rx_ver" localSheetId="1">Geometry!$D$49</definedName>
     <definedName name="stir_bar_L" localSheetId="1">Geometry!$D$50</definedName>
+    <definedName name="media_volume" localSheetId="1">Geometry!$D$85</definedName>
+    <definedName name="media_vol_warn" localSheetId="1">Geometry!$D$86</definedName>
+    <definedName name="depth_warn" localSheetId="1">Geometry!$D$87</definedName>
     <definedName name="etaF" localSheetId="2">Electrochemistry!$D$11</definedName>
     <definedName name="etaF_OER" localSheetId="2">Electrochemistry!$D$19</definedName>
     <definedName name="F_const" localSheetId="2">Electrochemistry!$D$8</definedName>
@@ -236,6 +244,7 @@
     <definedName name="DO_ss" localSheetId="4">'Mass Transfer'!$D$109</definedName>
     <definedName name="DO_ss_vs_opt" localSheetId="4">'Mass Transfer'!$D$110</definedName>
     <definedName name="DO_ss_vs_min" localSheetId="4">'Mass Transfer'!$D$111</definedName>
+    <definedName name="tip_warn" localSheetId="4">'Mass Transfer'!$D$112</definedName>
     <definedName name="CO2_cons" localSheetId="5">Dosing!$D$25</definedName>
     <definedName name="CO2_pulse" localSheetId="5">Dosing!$D$10</definedName>
     <definedName name="CO2_sd_ratio" localSheetId="5">Dosing!$D$14</definedName>
@@ -288,7 +297,7 @@
     <numFmt numFmtId="171" formatCode="0.0000000"/>
     <numFmt numFmtId="172" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -429,6 +438,14 @@
     </font>
     <font>
       <color rgb="FF000000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF0000FF"/>
+    </font>
+    <font>
+      <color rgb="FF0000FF"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="17">
@@ -708,7 +725,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -830,11 +847,20 @@
     <xf numFmtId="0" fontId="23" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="23" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="23" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="23" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="23" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="13">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -920,6 +946,20 @@
         <patternFill patternType="solid">
           <fgColor rgb="FF63BE7B"/>
           <bgColor rgb="FF63BE7B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1180,7 +1220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1300,6 +1340,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="59" t="inlineStr">
         <is>
@@ -1317,10 +1358,9 @@
         <f>'Mass Transfer'!$D$67</f>
         <v/>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>From Mass Transfer.</t>
-        </is>
+      <c r="E8" s="87">
+        <f>HYPERLINK("#'Mass Transfer'!D67","From Mass Transfer")</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -1333,10 +1373,9 @@
         <f>'Mass Transfer'!$D$68</f>
         <v/>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>From Mass Transfer.</t>
-        </is>
+      <c r="E9" s="87">
+        <f>HYPERLINK("#'Mass Transfer'!D68","From Mass Transfer")</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -1349,10 +1388,9 @@
         <f>'Mass Transfer'!$D$55</f>
         <v/>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>From Mass Transfer.</t>
-        </is>
+      <c r="E10" s="87">
+        <f>HYPERLINK("#'Mass Transfer'!D55","From Mass Transfer")</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -1365,10 +1403,9 @@
         <f>'Mass Transfer'!$D$56</f>
         <v/>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>From Mass Transfer.</t>
-        </is>
+      <c r="E11" s="87">
+        <f>HYPERLINK("#'Mass Transfer'!D56","From Mass Transfer")</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -1381,10 +1418,9 @@
         <f>Biology!$D$28</f>
         <v/>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>From Biology.</t>
-        </is>
+      <c r="E12" s="87">
+        <f>HYPERLINK("#Biology!D28","From Biology")</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -1397,10 +1433,9 @@
         <f>Dosing!$D$14</f>
         <v/>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>From Dosing.</t>
-        </is>
+      <c r="E13" s="87">
+        <f>HYPERLINK("#Dosing!D14","From Dosing")</f>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -1413,10 +1448,9 @@
         <f>Electrochemistry!$D$13</f>
         <v/>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>From Electrochemistry.</t>
-        </is>
+      <c r="E14" s="87">
+        <f>HYPERLINK("#Electrochemistry!D13","From Electrochemistry")</f>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -1429,10 +1463,9 @@
         <f>'Mass Transfer'!$D$35</f>
         <v/>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>From Mass Transfer.</t>
-        </is>
+      <c r="E15" s="87">
+        <f>HYPERLINK("#'Mass Transfer'!D35","From Mass Transfer")</f>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -1445,10 +1478,9 @@
         <f>'Mass Transfer'!$D$40</f>
         <v/>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>From Mass Transfer.</t>
-        </is>
+      <c r="E16" s="87">
+        <f>HYPERLINK("#'Mass Transfer'!D40","From Mass Transfer")</f>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -1461,10 +1493,9 @@
         <f>Dosing!$D$19</f>
         <v/>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>From Dosing.</t>
-        </is>
+      <c r="E17" s="87">
+        <f>HYPERLINK("#Dosing!D19","From Dosing")</f>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -1477,10 +1508,9 @@
         <f>'Mass Transfer'!$D$72</f>
         <v/>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>From Mass Transfer.</t>
-        </is>
+      <c r="E18" s="87">
+        <f>HYPERLINK("#'Mass Transfer'!D72","From Mass Transfer")</f>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -1493,10 +1523,9 @@
         <f>Biology!$D$37</f>
         <v/>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>From Biology.</t>
-        </is>
+      <c r="E19" s="87">
+        <f>HYPERLINK("#Biology!D37","From Biology")</f>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -1507,6 +1536,10 @@
       </c>
       <c r="D20" s="76">
         <f>Dosing!$D$41</f>
+        <v/>
+      </c>
+      <c r="E20" s="87">
+        <f>HYPERLINK("#Dosing!D41","From Dosing")</f>
         <v/>
       </c>
     </row>
@@ -1586,6 +1619,7 @@
       <c r="C30" s="28" t="n"/>
       <c r="D30" s="29" t="n"/>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="73" t="inlineStr">
         <is>
@@ -1661,40 +1695,393 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>LED intensity setpoint</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>led_intensity</t>
+        </is>
+      </c>
+      <c r="D37" s="88" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Stirrer rate (rpm)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>stir_rpm_set</t>
+        </is>
+      </c>
+      <c r="D38" s="88" t="n">
+        <v>500</v>
+      </c>
+    </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Steady-state DO (surface, mg/L)</t>
-        </is>
-      </c>
-      <c r="D39" s="83">
-        <f>'Mass Transfer'!$D$109</f>
-        <v/>
-      </c>
+          <t>Media volume (mL) - blank = recommended max</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>media_volume</t>
+        </is>
+      </c>
+      <c r="D39" s="89" t="n"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>DO vs organism optimum</t>
-        </is>
-      </c>
-      <c r="D40" s="83">
-        <f>'Mass Transfer'!$D$110</f>
-        <v/>
+          <t>Temperature (degC)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>temp_C</t>
+        </is>
+      </c>
+      <c r="D40" s="89" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>Ambient pressure (Pa)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>P_atm_set</t>
+        </is>
+      </c>
+      <c r="D41" s="89" t="n">
+        <v>101325</v>
+      </c>
+    </row>
+    <row r="42"/>
+    <row r="43">
+      <c r="A43" s="69" t="inlineStr">
+        <is>
+          <t>DO BAND (organism)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Steady-state DO (surface, mg/L)</t>
+        </is>
+      </c>
+      <c r="D44" s="80">
+        <f>'Mass Transfer'!$D$109</f>
+        <v/>
+      </c>
+      <c r="E44" s="87">
+        <f>HYPERLINK("#'Mass Transfer'!D109","From Mass Transfer")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>DO vs organism optimum</t>
+        </is>
+      </c>
+      <c r="D45" s="80">
+        <f>'Mass Transfer'!$D$110</f>
+        <v/>
+      </c>
+      <c r="E45" s="87">
+        <f>HYPERLINK("#'Mass Transfer'!D110","From Mass Transfer")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>DO vs organism minimum</t>
         </is>
       </c>
-      <c r="D41" s="83">
+      <c r="D46" s="80">
         <f>'Mass Transfer'!$D$111</f>
         <v/>
       </c>
+      <c r="E46" s="87">
+        <f>HYPERLINK("#'Mass Transfer'!D111","From Mass Transfer")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="69" t="inlineStr">
+        <is>
+          <t>Media-volume / depth / tip warnings</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Media vs max working</t>
+        </is>
+      </c>
+      <c r="D48" s="79">
+        <f>Geometry!$D$86</f>
+        <v/>
+      </c>
+      <c r="E48" s="87">
+        <f>HYPERLINK("#Geometry!D86","From Geometry")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Liquid vs usable depth</t>
+        </is>
+      </c>
+      <c r="D49" s="79">
+        <f>Geometry!$D$87</f>
+        <v/>
+      </c>
+      <c r="E49" s="87">
+        <f>HYPERLINK("#Geometry!D87","From Geometry")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Tip speed (m/s)</t>
+        </is>
+      </c>
+      <c r="D50" s="80">
+        <f>'Mass Transfer'!$D$45</f>
+        <v/>
+      </c>
+      <c r="E50" s="87">
+        <f>HYPERLINK("#'Mass Transfer'!D45","From Mass Transfer")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Tip-speed shear</t>
+        </is>
+      </c>
+      <c r="D51" s="80">
+        <f>'Mass Transfer'!$D$112</f>
+        <v/>
+      </c>
+      <c r="E51" s="87">
+        <f>HYPERLINK("#'Mass Transfer'!D112","From Mass Transfer")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52"/>
+    <row r="53">
+      <c r="A53" s="69" t="inlineStr">
+        <is>
+          <t>RANKED IMPROVEMENTS (by impact, with effort)</t>
+        </is>
+      </c>
+      <c r="B53" s="69" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="C53" s="69" t="inlineStr">
+        <is>
+          <t>Effort</t>
+        </is>
+      </c>
+      <c r="E53" s="69" t="inlineStr">
+        <is>
+          <t>Why it matters</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>1 Measure surface kLa (kL_surf)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>375% sensitivity; decides whether DO stays in the organism band</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2 Measure cathodic Faradaic efficiency (etaF)</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>sets the H2/O2 split and net O2; currently assumed 1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>3 Determine organism minimum DO</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>lower DO guardrail; currently a gap for every organism</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>4 Calibrate flow for each reactor used</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>each experiment; only ed04 calibrated so far</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>5 Confirm knallgas uptake ratio (H2:O2:CO2)</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>carbon/O2 balance; needs a growing culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>6 Measure sinter porosity grade</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>bubble size when sparger = sintered</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>7 Record lab ambient pressure</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Henry solubilities + gas volumes</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="D7:D20">
+    <cfRule type="expression" priority="1" dxfId="11">
+      <formula>OR(ISNUMBER(SEARCH("RISK",D7)),ISNUMBER(SEARCH("OVER",D7)),ISNUMBER(SEARCH("BELOW",D7)),ISNUMBER(SEARCH("EXCEED",D7)),ISNUMBER(SEARCH("NO CALIB",D7)),ISNUMBER(SEARCH("NEAREST",D7)),ISNUMBER(SEARCH("EXPLOSIVE",D7)),ISNUMBER(SEARCH("LOW",D7)),ISNUMBER(SEARCH("TIGHT",D7)),ISNUMBER(SEARCH("insufficient",D7)))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="12">
+      <formula>OR(ISNUMBER(SEARCH("OK",D7)),ISNUMBER(SEARCH("calibrated",D7)),ISNUMBER(SEARCH("under optimum",D7)),ISNUMBER(SEARCH("above min",D7)),ISNUMBER(SEARCH("exact",D7)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D44:D51">
+    <cfRule type="expression" priority="3" dxfId="11">
+      <formula>OR(ISNUMBER(SEARCH("RISK",D44)),ISNUMBER(SEARCH("OVER",D44)),ISNUMBER(SEARCH("BELOW",D44)),ISNUMBER(SEARCH("EXCEED",D44)),ISNUMBER(SEARCH("NO CALIB",D44)),ISNUMBER(SEARCH("NEAREST",D44)),ISNUMBER(SEARCH("EXPLOSIVE",D44)),ISNUMBER(SEARCH("LOW",D44)),ISNUMBER(SEARCH("TIGHT",D44)),ISNUMBER(SEARCH("insufficient",D44)))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="12">
+      <formula>OR(ISNUMBER(SEARCH("OK",D44)),ISNUMBER(SEARCH("calibrated",D44)),ISNUMBER(SEARCH("under optimum",D44)),ISNUMBER(SEARCH("above min",D44)),ISNUMBER(SEARCH("exact",D44)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="5">
     <dataValidation sqref="D5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
       <formula1>"0,1,2,3,4,5"</formula1>
@@ -1724,7 +2111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I83"/>
+  <dimension ref="A1:I87"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2626,8 +3013,8 @@
           <t>mL</t>
         </is>
       </c>
-      <c r="D36" s="38">
-        <f>ROUND(V_max-disp_tot,0)</f>
+      <c r="D36" s="90">
+        <f>IF(media_volume&gt;0,media_volume,ROUND(V_max-disp_tot,0))</f>
         <v/>
       </c>
       <c r="E36" s="14" t="inlineStr">
@@ -2868,6 +3255,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="64" t="inlineStr">
         <is>
@@ -3216,6 +3604,7 @@
         </is>
       </c>
     </row>
+    <row r="75"/>
     <row r="76">
       <c r="A76" s="73" t="inlineStr">
         <is>
@@ -3402,6 +3791,7 @@
         <v>6</v>
       </c>
     </row>
+    <row r="82"/>
     <row r="83">
       <c r="A83" s="72" t="inlineStr">
         <is>
@@ -3409,7 +3799,64 @@
         </is>
       </c>
     </row>
+    <row r="84"/>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>(import) Media volume (set)</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>media_volume</t>
+        </is>
+      </c>
+      <c r="D85" s="79">
+        <f>Summary!$D$39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Media vs max working volume</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>media_vol_warn</t>
+        </is>
+      </c>
+      <c r="D86" s="80">
+        <f>IF(V_charge&gt;V_max,"MEDIA &gt; MAX WORKING VOLUME","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Liquid level vs usable depth</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>depth_warn</t>
+        </is>
+      </c>
+      <c r="D87" s="80">
+        <f>IF(h_actual&gt;D_int,"LIQUID OVER USABLE DEPTH","OK")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="D86:D87">
+    <cfRule type="expression" priority="1" dxfId="11">
+      <formula>OR(ISNUMBER(SEARCH("RISK",D86)),ISNUMBER(SEARCH("OVER",D86)),ISNUMBER(SEARCH("BELOW",D86)),ISNUMBER(SEARCH("EXCEED",D86)),ISNUMBER(SEARCH("NO CALIB",D86)),ISNUMBER(SEARCH("NEAREST",D86)),ISNUMBER(SEARCH("EXPLOSIVE",D86)),ISNUMBER(SEARCH("LOW",D86)),ISNUMBER(SEARCH("TIGHT",D86)),ISNUMBER(SEARCH("insufficient",D86)))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="12">
+      <formula>OR(ISNUMBER(SEARCH("OK",D86)),ISNUMBER(SEARCH("calibrated",D86)),ISNUMBER(SEARCH("under optimum",D86)),ISNUMBER(SEARCH("above min",D86)),ISNUMBER(SEARCH("exact",D86)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3479,8 +3926,9 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D3" s="39" t="n">
-        <v>3</v>
+      <c r="D3" s="91">
+        <f>Summary!$D$37</f>
+        <v/>
       </c>
       <c r="E3" s="10" t="inlineStr">
         <is>
@@ -3973,6 +4421,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="64" t="inlineStr">
         <is>
@@ -4058,6 +4507,8 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="73" t="inlineStr">
         <is>
@@ -4235,6 +4686,7 @@
         <v>2</v>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="72" t="inlineStr">
         <is>
@@ -4242,6 +4694,7 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
@@ -4531,8 +4984,9 @@
           <t>°C</t>
         </is>
       </c>
-      <c r="D10" s="31" t="n">
-        <v>30</v>
+      <c r="D10" s="92">
+        <f>Summary!$D$40</f>
+        <v/>
       </c>
       <c r="E10" s="10" t="inlineStr">
         <is>
@@ -4582,8 +5036,9 @@
           <t>Pa</t>
         </is>
       </c>
-      <c r="D12" s="30" t="n">
-        <v>101325</v>
+      <c r="D12" s="79">
+        <f>Summary!$D$41</f>
+        <v/>
       </c>
       <c r="E12" s="10" t="inlineStr">
         <is>
@@ -5230,6 +5685,7 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
     <row r="39">
       <c r="A39" s="64" t="inlineStr">
         <is>
@@ -5315,6 +5771,8 @@
         </is>
       </c>
     </row>
+    <row r="43"/>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="73" t="inlineStr">
         <is>
@@ -5538,6 +5996,7 @@
         </is>
       </c>
     </row>
+    <row r="53"/>
     <row r="54">
       <c r="A54" s="73" t="inlineStr">
         <is>
@@ -5708,7 +6167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E111"/>
+  <dimension ref="A1:E112"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6791,8 +7250,9 @@
           <t>1/min</t>
         </is>
       </c>
-      <c r="D43" s="52" t="n">
-        <v>500</v>
+      <c r="D43" s="93">
+        <f>Summary!$D$38</f>
+        <v/>
       </c>
       <c r="E43" s="25" t="inlineStr">
         <is>
@@ -7629,6 +8089,7 @@
         </is>
       </c>
     </row>
+    <row r="76"/>
     <row r="77">
       <c r="A77" s="64" t="inlineStr">
         <is>
@@ -8198,7 +8659,7 @@
           <t>0-5</t>
         </is>
       </c>
-      <c r="D99">
+      <c r="D99" s="94">
         <f>Summary!$D$5</f>
         <v/>
       </c>
@@ -8234,6 +8695,7 @@
         </is>
       </c>
     </row>
+    <row r="101"/>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
@@ -8324,6 +8786,7 @@
         <v/>
       </c>
     </row>
+    <row r="107"/>
     <row r="108">
       <c r="A108" s="69" t="inlineStr">
         <is>
@@ -8377,6 +8840,27 @@
       <c r="D111" s="80">
         <f>IF(ISNUMBER(DO_min),IF(DO_ss&gt;=DO_min,"above minimum","BELOW MINIMUM"),"minimum DO unknown - measure")</f>
         <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Tip-speed shear flag (&lt;1.5 m/s)</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>tip_warn</t>
+        </is>
+      </c>
+      <c r="D112" s="80">
+        <f>IF(tip_speed&gt;1.5,"TIP SPEED &gt; 1.5 m/s","OK")</f>
+        <v/>
+      </c>
+      <c r="E112" s="95" t="inlineStr">
+        <is>
+          <t>Conservative shear limit: &lt;1.5 m/s impeller-tip velocity recommended to avoid adverse cell-growth effects (BioProcess International, cell-culture norm); precautionary for robust HOB.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -8479,6 +8963,14 @@
       <formula>"TIGHT"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="D110:D112">
+    <cfRule type="expression" priority="14" dxfId="11">
+      <formula>OR(ISNUMBER(SEARCH("RISK",D110)),ISNUMBER(SEARCH("OVER",D110)),ISNUMBER(SEARCH("BELOW",D110)),ISNUMBER(SEARCH("EXCEED",D110)),ISNUMBER(SEARCH("NO CALIB",D110)),ISNUMBER(SEARCH("NEAREST",D110)),ISNUMBER(SEARCH("EXPLOSIVE",D110)),ISNUMBER(SEARCH("LOW",D110)),ISNUMBER(SEARCH("TIGHT",D110)),ISNUMBER(SEARCH("insufficient",D110)))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="12">
+      <formula>OR(ISNUMBER(SEARCH("OK",D110)),ISNUMBER(SEARCH("calibrated",D110)),ISNUMBER(SEARCH("under optimum",D110)),ISNUMBER(SEARCH("above min",D110)),ISNUMBER(SEARCH("exact",D110)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8968,6 +9460,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="64" t="inlineStr">
         <is>
@@ -9235,6 +9728,7 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="69" t="inlineStr">
         <is>
@@ -9426,6 +9920,20 @@
     <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
       <formula>"LOW"</formula>
     </cfRule>
+    <cfRule type="expression" priority="4" dxfId="11">
+      <formula>OR(ISNUMBER(SEARCH("RISK",D19)),ISNUMBER(SEARCH("OVER",D19)),ISNUMBER(SEARCH("BELOW",D19)),ISNUMBER(SEARCH("EXCEED",D19)),ISNUMBER(SEARCH("NO CALIB",D19)),ISNUMBER(SEARCH("NEAREST",D19)),ISNUMBER(SEARCH("EXPLOSIVE",D19)),ISNUMBER(SEARCH("LOW",D19)),ISNUMBER(SEARCH("TIGHT",D19)),ISNUMBER(SEARCH("insufficient",D19)))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="12">
+      <formula>OR(ISNUMBER(SEARCH("OK",D19)),ISNUMBER(SEARCH("calibrated",D19)),ISNUMBER(SEARCH("under optimum",D19)),ISNUMBER(SEARCH("above min",D19)),ISNUMBER(SEARCH("exact",D19)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D41">
+    <cfRule type="expression" priority="6" dxfId="11">
+      <formula>OR(ISNUMBER(SEARCH("RISK",D41)),ISNUMBER(SEARCH("OVER",D41)),ISNUMBER(SEARCH("BELOW",D41)),ISNUMBER(SEARCH("EXCEED",D41)),ISNUMBER(SEARCH("NO CALIB",D41)),ISNUMBER(SEARCH("NEAREST",D41)),ISNUMBER(SEARCH("EXPLOSIVE",D41)),ISNUMBER(SEARCH("LOW",D41)),ISNUMBER(SEARCH("TIGHT",D41)),ISNUMBER(SEARCH("insufficient",D41)))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="12">
+      <formula>OR(ISNUMBER(SEARCH("OK",D41)),ISNUMBER(SEARCH("calibrated",D41)),ISNUMBER(SEARCH("under optimum",D41)),ISNUMBER(SEARCH("above min",D41)),ISNUMBER(SEARCH("exact",D41)))</formula>
+    </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="D58" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
@@ -9444,7 +9952,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q76"/>
+  <dimension ref="A1:Q75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="9"/>
@@ -10791,7 +11299,6 @@
     <row r="75">
       <c r="A75" s="73" t="n"/>
     </row>
-    <row r="76"/>
   </sheetData>
   <conditionalFormatting sqref="H5:H46">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
model(modular): expose both schedule regimes (O2-limited vs carbon-limited) + verdict
The optimal interval depends on whether surface stripping or sparging removes O2:
- O2-limited (conservative, current model optimum): ~1.4 min pulse-to-pulse
- carbon-limited (if surface stripping handles O2, as DO_ss~1.9 mg/L suggests): ~178 min
The 100x gap is resolved by measuring kL_surf. Added spg_int_carbon + a regime verdict cell,
surfaced on Summary, so neither bound is presented as definitive on its own.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel-modular.xlsx
+++ b/Media/electroPioreactorGasModel-modular.xlsx
@@ -245,6 +245,8 @@
     <definedName name="DO_ss_vs_opt" localSheetId="4">'Mass Transfer'!$D$110</definedName>
     <definedName name="DO_ss_vs_min" localSheetId="4">'Mass Transfer'!$D$111</definedName>
     <definedName name="tip_warn" localSheetId="4">'Mass Transfer'!$D$112</definedName>
+    <definedName name="spg_int_carbon" localSheetId="4">'Mass Transfer'!$D$113</definedName>
+    <definedName name="sched_regime" localSheetId="4">'Mass Transfer'!$D$114</definedName>
     <definedName name="CO2_cons" localSheetId="5">Dosing!$D$25</definedName>
     <definedName name="CO2_pulse" localSheetId="5">Dosing!$D$10</definedName>
     <definedName name="CO2_sd_ratio" localSheetId="5">Dosing!$D$14</definedName>
@@ -1220,7 +1222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1340,7 +1342,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="59" t="inlineStr">
         <is>
@@ -1619,7 +1620,6 @@
       <c r="C30" s="28" t="n"/>
       <c r="D30" s="29" t="n"/>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="73" t="inlineStr">
         <is>
@@ -1768,7 +1768,6 @@
         <v>101325</v>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="69" t="inlineStr">
         <is>
@@ -1888,7 +1887,6 @@
         <v/>
       </c>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="69" t="inlineStr">
         <is>
@@ -2063,6 +2061,50 @@
         <is>
           <t>Henry solubilities + gas volumes</t>
         </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="69" t="inlineStr">
+        <is>
+          <t>SCHEDULE REGIME</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Interval - O2-limited (conservative, model optimum, min)</t>
+        </is>
+      </c>
+      <c r="D63" s="80">
+        <f>'Mass Transfer'!$D$68</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Interval - carbon-limited if O2 handled by surface (min)</t>
+        </is>
+      </c>
+      <c r="D64" s="80">
+        <f>'Mass Transfer'!$D$113</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Which regime</t>
+        </is>
+      </c>
+      <c r="D65" s="80">
+        <f>'Mass Transfer'!$D$114</f>
+        <v/>
+      </c>
+      <c r="E65">
+        <f>'Mass Transfer'!$E$114</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -3255,7 +3297,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="64" t="inlineStr">
         <is>
@@ -3604,7 +3645,6 @@
         </is>
       </c>
     </row>
-    <row r="75"/>
     <row r="76">
       <c r="A76" s="73" t="inlineStr">
         <is>
@@ -3791,7 +3831,6 @@
         <v>6</v>
       </c>
     </row>
-    <row r="82"/>
     <row r="83">
       <c r="A83" s="72" t="inlineStr">
         <is>
@@ -3799,7 +3838,6 @@
         </is>
       </c>
     </row>
-    <row r="84"/>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
@@ -4421,7 +4459,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="64" t="inlineStr">
         <is>
@@ -4507,8 +4544,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="73" t="inlineStr">
         <is>
@@ -4686,7 +4721,6 @@
         <v>2</v>
       </c>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="72" t="inlineStr">
         <is>
@@ -4694,7 +4728,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
@@ -5685,7 +5718,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="A39" s="64" t="inlineStr">
         <is>
@@ -5771,8 +5803,6 @@
         </is>
       </c>
     </row>
-    <row r="43"/>
-    <row r="44"/>
     <row r="45">
       <c r="A45" s="73" t="inlineStr">
         <is>
@@ -5996,7 +6026,6 @@
         </is>
       </c>
     </row>
-    <row r="53"/>
     <row r="54">
       <c r="A54" s="73" t="inlineStr">
         <is>
@@ -6167,7 +6196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E112"/>
+  <dimension ref="A1:E114"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8089,7 +8118,6 @@
         </is>
       </c>
     </row>
-    <row r="76"/>
     <row r="77">
       <c r="A77" s="64" t="inlineStr">
         <is>
@@ -8695,7 +8723,6 @@
         </is>
       </c>
     </row>
-    <row r="101"/>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
@@ -8786,7 +8813,6 @@
         <v/>
       </c>
     </row>
-    <row r="107"/>
     <row r="108">
       <c r="A108" s="69" t="inlineStr">
         <is>
@@ -8860,6 +8886,43 @@
       <c r="E112" s="95" t="inlineStr">
         <is>
           <t>Conservative shear limit: &lt;1.5 m/s impeller-tip velocity recommended to avoid adverse cell-growth effects (BioProcess International, cell-culture norm); precautionary for robust HOB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Interval if surface stripping handles O2 (carbon-limited)</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>spg_int_carbon</t>
+        </is>
+      </c>
+      <c r="D113" s="80">
+        <f>spg_dur_opt/(60*duty_carbon)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Schedule regime (which interval applies)</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>sched_regime</t>
+        </is>
+      </c>
+      <c r="D114" s="80">
+        <f>IF(ISNUMBER(DO_ss),IF(DO_ss&lt;DO_impair,"Surface stripping holds DO under impairment - sparge is CARBON-limited (long interval); the O2-limited interval is the conservative fallback until kL_surf is measured","Surface stripping insufficient - sparge must vent O2 - use the O2-limited interval"),"organism DO unknown")</f>
+        <v/>
+      </c>
+      <c r="E114" s="95" t="inlineStr">
+        <is>
+          <t>Resolved by measuring kL_surf (improvement #1).</t>
         </is>
       </c>
     </row>
@@ -9460,7 +9523,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="64" t="inlineStr">
         <is>
@@ -9728,7 +9790,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" s="69" t="inlineStr">
         <is>
@@ -11251,7 +11312,6 @@
     <row r="47">
       <c r="B47" s="66" t="n"/>
     </row>
-    <row r="48"/>
     <row r="49">
       <c r="A49" s="73" t="n"/>
     </row>
@@ -11268,34 +11328,15 @@
     <row r="52">
       <c r="A52" s="72" t="n"/>
     </row>
-    <row r="53"/>
     <row r="54">
       <c r="A54" s="73" t="n"/>
     </row>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="72" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="72" t="n"/>
     </row>
-    <row r="74"/>
     <row r="75">
       <c r="A75" s="73" t="n"/>
     </row>

</xml_diff>

<commit_message>
model(modular): fold Dosing tab into Mass Transfer (no behavioural change)
- 16 Dosing-only cells moved into a 'CO2 DOSING & SCHEDULE (folded)' block on Mass Transfer (rows 116-132), each keeping its defined name and verbatim formula
- the 8 Mass Transfer cells that imported from Dosing now carry the real formula/constant in place (Q_CO2, pulse_floor, R_gas, M_CO2, nCO2_rate, CO2_supply, duty, flush_factor); 10 redundant Dosing imports dropped
- external refs repointed (Electrochemistry R_gas; Summary CO2_sd_ratio/dur_ok/cal_warning + their hyperlinks); Dosing sheet deleted
- independently verified: no #REF, all names resolve to their col-B-labelled cell, 5 dropdowns intact, every headline number unchanged

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel-modular.xlsx
+++ b/Media/electroPioreactorGasModel-modular.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="580" windowWidth="20400" windowHeight="18060" tabRatio="500" firstSheet="0" activeTab="6" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="580" windowWidth="20400" windowHeight="18060" tabRatio="500" firstSheet="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -11,8 +11,7 @@
     <sheet name="Electrochemistry" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Biology" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Mass Transfer" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Dosing" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="CO2 flows" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="CO2 flows" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="por_grade" localSheetId="0">Summary!$D$5</definedName>
@@ -247,40 +246,22 @@
     <definedName name="tip_warn" localSheetId="4">'Mass Transfer'!$D$112</definedName>
     <definedName name="spg_int_carbon" localSheetId="4">'Mass Transfer'!$D$113</definedName>
     <definedName name="sched_regime" localSheetId="4">'Mass Transfer'!$D$114</definedName>
-    <definedName name="CO2_cons" localSheetId="5">Dosing!$D$25</definedName>
-    <definedName name="CO2_pulse" localSheetId="5">Dosing!$D$10</definedName>
-    <definedName name="CO2_sd_ratio" localSheetId="5">Dosing!$D$14</definedName>
-    <definedName name="CO2_supply" localSheetId="5">Dosing!$D$13</definedName>
-    <definedName name="dur_ok" localSheetId="5">Dosing!$D$19</definedName>
-    <definedName name="duty" localSheetId="5">Dosing!$D$15</definedName>
-    <definedName name="M_CO2" localSheetId="5">Dosing!$D$8</definedName>
-    <definedName name="nCO2_rate" localSheetId="5">Dosing!$D$9</definedName>
-    <definedName name="O2_accum" localSheetId="5">Dosing!$D$16</definedName>
-    <definedName name="O2_excess" localSheetId="5">Dosing!$D$22</definedName>
-    <definedName name="O2_strip_pulse" localSheetId="5">Dosing!$D$17</definedName>
-    <definedName name="P_atm" localSheetId="5">Dosing!$D$24</definedName>
-    <definedName name="pulse_floor" localSheetId="5">Dosing!$D$6</definedName>
-    <definedName name="pulses_d" localSheetId="5">Dosing!$D$12</definedName>
-    <definedName name="pulses_h" localSheetId="5">Dosing!$D$11</definedName>
-    <definedName name="Q_CO2" localSheetId="5">Dosing!$D$3</definedName>
-    <definedName name="R_gas" localSheetId="5">Dosing!$D$7</definedName>
-    <definedName name="sched_bal" localSheetId="5">Dosing!$D$18</definedName>
-    <definedName name="sched_mode" localSheetId="5">Dosing!$D$27</definedName>
-    <definedName name="spg_dur" localSheetId="5">Dosing!$D$4</definedName>
-    <definedName name="spg_dur_man" localSheetId="5">Dosing!$D$30</definedName>
-    <definedName name="spg_dur_opt" localSheetId="5">Dosing!$D$28</definedName>
-    <definedName name="spg_int" localSheetId="5">Dosing!$D$5</definedName>
-    <definedName name="spg_int_man" localSheetId="5">Dosing!$D$26</definedName>
-    <definedName name="spg_int_opt" localSheetId="5">Dosing!$D$31</definedName>
-    <definedName name="strip_sparge" localSheetId="5">Dosing!$D$29</definedName>
-    <definedName name="T_K" localSheetId="5">Dosing!$D$23</definedName>
-    <definedName name="Reactor" localSheetId="5">Dosing!$D$34</definedName>
-    <definedName name="flush_factor" localSheetId="5">Dosing!$D$35</definedName>
-    <definedName name="latest_date" localSheetId="5">Dosing!$D$36</definedName>
-    <definedName name="flowrate_cal" localSheetId="5">Dosing!$D$37</definedName>
-    <definedName name="min_sparge_cal" localSheetId="5">Dosing!$D$38</definedName>
-    <definedName name="cal_warning" localSheetId="5">Dosing!$D$41</definedName>
-    <definedName name="has_cal" localSheetId="5">Dosing!$D$39</definedName>
+    <definedName name="Reactor" localSheetId="4">'Mass Transfer'!$D$117</definedName>
+    <definedName name="latest_date" localSheetId="4">'Mass Transfer'!$D$118</definedName>
+    <definedName name="flowrate_cal" localSheetId="4">'Mass Transfer'!$D$119</definedName>
+    <definedName name="min_sparge_cal" localSheetId="4">'Mass Transfer'!$D$120</definedName>
+    <definedName name="has_cal" localSheetId="4">'Mass Transfer'!$D$121</definedName>
+    <definedName name="cal_warning" localSheetId="4">'Mass Transfer'!$D$122</definedName>
+    <definedName name="spg_dur" localSheetId="4">'Mass Transfer'!$D$123</definedName>
+    <definedName name="spg_int" localSheetId="4">'Mass Transfer'!$D$124</definedName>
+    <definedName name="CO2_pulse" localSheetId="4">'Mass Transfer'!$D$125</definedName>
+    <definedName name="pulses_h" localSheetId="4">'Mass Transfer'!$D$126</definedName>
+    <definedName name="pulses_d" localSheetId="4">'Mass Transfer'!$D$127</definedName>
+    <definedName name="CO2_sd_ratio" localSheetId="4">'Mass Transfer'!$D$128</definedName>
+    <definedName name="O2_accum" localSheetId="4">'Mass Transfer'!$D$129</definedName>
+    <definedName name="O2_strip_pulse" localSheetId="4">'Mass Transfer'!$D$130</definedName>
+    <definedName name="sched_bal" localSheetId="4">'Mass Transfer'!$D$131</definedName>
+    <definedName name="dur_ok" localSheetId="4">'Mass Transfer'!$D$132</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
@@ -299,7 +280,7 @@
     <numFmt numFmtId="171" formatCode="0.0000000"/>
     <numFmt numFmtId="172" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -449,6 +430,9 @@
       <color rgb="FF0000FF"/>
       <u val="single"/>
     </font>
+    <font>
+      <color rgb="FF7030A0"/>
+    </font>
   </fonts>
   <fills count="17">
     <fill>
@@ -541,7 +525,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -723,11 +707,12 @@
         <color theme="6"/>
       </bottom>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -858,6 +843,8 @@
     <xf numFmtId="164" fontId="23" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1430,12 +1417,12 @@
           <t>CO₂ supply:demand</t>
         </is>
       </c>
-      <c r="D13" s="62">
-        <f>Dosing!$D$14</f>
+      <c r="D13" s="79">
+        <f>'Mass Transfer'!$D$128</f>
         <v/>
       </c>
       <c r="E13" s="87">
-        <f>HYPERLINK("#Dosing!D14","From Dosing")</f>
+        <f>HYPERLINK("#'Mass Transfer'!D128","From Mass Transfer")</f>
         <v/>
       </c>
     </row>
@@ -1490,12 +1477,12 @@
           <t>Pulse≥floor</t>
         </is>
       </c>
-      <c r="D17" s="62">
-        <f>Dosing!$D$19</f>
+      <c r="D17" s="79">
+        <f>'Mass Transfer'!$D$132</f>
         <v/>
       </c>
       <c r="E17" s="87">
-        <f>HYPERLINK("#Dosing!D19","From Dosing")</f>
+        <f>HYPERLINK("#'Mass Transfer'!D132","From Mass Transfer")</f>
         <v/>
       </c>
     </row>
@@ -1535,12 +1522,12 @@
           <t>Calibration source</t>
         </is>
       </c>
-      <c r="D20" s="76">
-        <f>Dosing!$D$41</f>
+      <c r="D20" s="79">
+        <f>'Mass Transfer'!$D$122</f>
         <v/>
       </c>
       <c r="E20" s="87">
-        <f>HYPERLINK("#Dosing!D41","From Dosing")</f>
+        <f>HYPERLINK("#'Mass Transfer'!D122","From Mass Transfer")</f>
         <v/>
       </c>
     </row>
@@ -4535,7 +4522,7 @@
         </is>
       </c>
       <c r="D27" s="62">
-        <f>Dosing!$D$7</f>
+        <f>'Mass Transfer'!$D$87</f>
         <v/>
       </c>
       <c r="E27" t="inlineStr">
@@ -6196,7 +6183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E114"/>
+  <dimension ref="A1:E132"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8310,7 +8297,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>(import) Min reliable pulse (solenoid floor)</t>
+          <t>Min reliable pulse (solenoid floor)</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -8323,8 +8310,8 @@
           <t>s</t>
         </is>
       </c>
-      <c r="D85" s="62">
-        <f>Dosing!$D$6</f>
+      <c r="D85" s="96">
+        <f>min_sparge_cal</f>
         <v/>
       </c>
       <c r="E85" t="inlineStr">
@@ -8336,7 +8323,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>(import) Average CO₂ supply rate</t>
+          <t>Average CO₂ supply rate</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -8349,8 +8336,8 @@
           <t>mol/h</t>
         </is>
       </c>
-      <c r="D86" s="62">
-        <f>Dosing!$D$13</f>
+      <c r="D86" s="96">
+        <f>CO2_pulse*pulses_h</f>
         <v/>
       </c>
       <c r="E86" t="inlineStr">
@@ -8362,7 +8349,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>(import) Ideal gas constant</t>
+          <t>Ideal gas constant</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -8375,9 +8362,8 @@
           <t>J/mol/K</t>
         </is>
       </c>
-      <c r="D87" s="62">
-        <f>Dosing!$D$7</f>
-        <v/>
+      <c r="D87" s="97" t="n">
+        <v>8.314462618</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -8388,7 +8374,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>(import) CO₂ volumetric flow rate</t>
+          <t>CO₂ volumetric flow rate</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -8401,8 +8387,8 @@
           <t>mL/min</t>
         </is>
       </c>
-      <c r="D88" s="62">
-        <f>Dosing!$D$3</f>
+      <c r="D88" s="96">
+        <f>flowrate_cal*60</f>
         <v/>
       </c>
       <c r="E88" t="inlineStr">
@@ -8414,7 +8400,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>(import) Molar mass CO₂</t>
+          <t>Molar mass CO₂</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -8427,9 +8413,8 @@
           <t>g/mol</t>
         </is>
       </c>
-      <c r="D89" s="62">
-        <f>Dosing!$D$8</f>
-        <v/>
+      <c r="D89" s="97" t="n">
+        <v>44.0095</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -8440,7 +8425,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>(import) CO₂ molar flow during sparge</t>
+          <t>CO₂ molar flow during sparge</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -8453,8 +8438,8 @@
           <t>mol/s</t>
         </is>
       </c>
-      <c r="D90" s="62">
-        <f>Dosing!$D$9</f>
+      <c r="D90" s="96">
+        <f>P_atm*(Q_CO2/1000000/60)/(R_gas*T_K)</f>
         <v/>
       </c>
       <c r="E90" t="inlineStr">
@@ -8466,7 +8451,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>(import) Sparge duty cycle</t>
+          <t>Sparge duty cycle</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -8479,8 +8464,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D91" s="62">
-        <f>Dosing!$D$15</f>
+      <c r="D91" s="96">
+        <f>spg_dur/(spg_int*60)</f>
         <v/>
       </c>
       <c r="E91" t="inlineStr">
@@ -8726,7 +8711,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>(import) CO2 per pulse (headspace vols)</t>
+          <t>CO2 per pulse (headspace volumes)</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -8739,9 +8724,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D102">
-        <f>Dosing!$D$35</f>
-        <v/>
+      <c r="D102" s="97" t="n">
+        <v>1</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -8924,6 +8908,269 @@
         <is>
           <t>Resolved by measuring kL_surf (improvement #1).</t>
         </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="69" t="inlineStr">
+        <is>
+          <t>CO₂ DOSING &amp; SCHEDULE (folded from Dosing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Reactor (calibration key)</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Reactor</t>
+        </is>
+      </c>
+      <c r="D117" s="79">
+        <f>Summary!$D$33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>latest calibration date</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>latest_date</t>
+        </is>
+      </c>
+      <c r="D118" s="80">
+        <f>SUMPRODUCT(MAX(('CO2 flows'!$A$4:$A$200=Reactor)*('CO2 flows'!$J$4:$J$200&gt;0)*'CO2 flows'!$B$4:$B$200))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>flowrate (calibrated)</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>flowrate_cal</t>
+        </is>
+      </c>
+      <c r="D119" s="80">
+        <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$200=Reactor)*('CO2 flows'!$B$4:$B$200=latest_date)*'CO2 flows'!$J$4:$J$200)/MAX(1,SUMPRODUCT(('CO2 flows'!$A$4:$A$200=Reactor)*('CO2 flows'!$B$4:$B$200=latest_date)*('CO2 flows'!$J$4:$J$200&gt;0)*1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>min sparge (calibrated)</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>min_sparge_cal</t>
+        </is>
+      </c>
+      <c r="D120" s="80">
+        <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$200=Reactor)*('CO2 flows'!$B$4:$B$200=latest_date)*'CO2 flows'!$I$4:$I$200)/MAX(1,SUMPRODUCT(('CO2 flows'!$A$4:$A$200=Reactor)*('CO2 flows'!$B$4:$B$200=latest_date)*('CO2 flows'!$J$4:$J$200&gt;0)*1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>reactor has a calibration row?</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>has_cal</t>
+        </is>
+      </c>
+      <c r="D121" s="80">
+        <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$200=Reactor)*('CO2 flows'!$J$4:$J$200&gt;0)*1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>calibration source</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>cal_warning</t>
+        </is>
+      </c>
+      <c r="D122" s="80">
+        <f>IF(has_cal&gt;0,"calibrated: "&amp;Reactor,"NO CALIBRATION for "&amp;Reactor&amp;" - add a row in CO2 flows with nominal flowrate + minimum sparge")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Sparge duration per pulse</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>spg_dur</t>
+        </is>
+      </c>
+      <c r="D123" s="80">
+        <f>IF(sched_mode="Optimal",spg_dur_opt,IF(sched_mode="Manual",spg_dur_man,NA()))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Sparge interval</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>spg_int</t>
+        </is>
+      </c>
+      <c r="D124" s="80">
+        <f>IF(sched_mode="Optimal",spg_int_opt,IF(sched_mode="Manual",spg_int_man,NA()))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>CO₂ per pulse</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>CO2_pulse</t>
+        </is>
+      </c>
+      <c r="D125" s="80">
+        <f>nCO2_rate*spg_dur</f>
+        <v/>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Pulses per hour</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>pulses_h</t>
+        </is>
+      </c>
+      <c r="D126" s="80">
+        <f>60/spg_int</f>
+        <v/>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Pulses per day</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>pulses_d</t>
+        </is>
+      </c>
+      <c r="D127" s="80">
+        <f>pulses_h*24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>CO₂ supply : carbon demand</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>CO2_sd_ratio</t>
+        </is>
+      </c>
+      <c r="D128" s="80">
+        <f>IF(CO2_cons&gt;0,CO2_supply/CO2_cons,NA())</f>
+        <v/>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>O₂ accumulated per interval</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>O2_accum</t>
+        </is>
+      </c>
+      <c r="D129" s="80">
+        <f>O2_excess/60*spg_int</f>
+        <v/>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>O₂ removable per pulse</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>O2_strip_pulse</t>
+        </is>
+      </c>
+      <c r="D130" s="80">
+        <f>strip_sparge/3600*spg_dur</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Per-pulse balance</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>sched_bal</t>
+        </is>
+      </c>
+      <c r="D131" s="80">
+        <f>IF(O2_accum&gt;0,O2_strip_pulse/O2_accum,NA())</f>
+        <v/>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Duration floor check</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>dur_ok</t>
+        </is>
+      </c>
+      <c r="D132" s="80">
+        <f>IF(spg_dur&gt;=pulse_floor,"OK","LOW")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -9045,974 +9292,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="57" t="inlineStr">
-        <is>
-          <t>CO₂ DOSING &amp; SCHEDULE</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="58" t="inlineStr">
-        <is>
-          <t>Parameter</t>
-        </is>
-      </c>
-      <c r="B2" s="58" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C2" s="58" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="D2" s="58" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="E2" s="58" t="inlineStr">
-        <is>
-          <t>Source / assumption</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>CO₂ volumetric flow rate</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>Q_CO2</t>
-        </is>
-      </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>mL/min</t>
-        </is>
-      </c>
-      <c r="D3" s="31">
-        <f>flowrate_cal*60</f>
-        <v/>
-      </c>
-      <c r="E3" s="10" t="inlineStr">
-        <is>
-          <t>Needle-valve setting at ~atmospheric surface. Input.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>Sparge duration per pulse</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>spg_dur</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="D4" s="32">
-        <f>IF(sched_mode="Optimal",spg_dur_opt,IF(sched_mode="Manual",spg_dur_man,NA()))</f>
-        <v/>
-      </c>
-      <c r="E4" s="10" t="inlineStr">
-        <is>
-          <t>Pulse duration ACTUALLY USED. Driven by §14: Manual→spg_dur_man, Optimal→computed optimum.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Sparge interval</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>spg_int</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>min</t>
-        </is>
-      </c>
-      <c r="D5" s="32">
-        <f>IF(sched_mode="Optimal",spg_int_opt,IF(sched_mode="Manual",spg_int_man,NA()))</f>
-        <v/>
-      </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>Sparge interval ACTUALLY USED. Driven by §14: Manual→spg_int_man, Optimal→computed optimum.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Min reliable pulse (solenoid floor)</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>pulse_floor</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="D6" s="24">
-        <f>min_sparge_cal</f>
-        <v/>
-      </c>
-      <c r="E6" s="15" t="inlineStr">
-        <is>
-          <t>Smallest dependable actuation. Provisional - characterise.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Ideal gas constant</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>R_gas</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>J/mol/K</t>
-        </is>
-      </c>
-      <c r="D7" s="47" t="n">
-        <v>8.314462618</v>
-      </c>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>NIST CODATA (exact, SI 2019).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Molar mass CO₂</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>M_CO2</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>g/mol</t>
-        </is>
-      </c>
-      <c r="D8" s="48" t="n">
-        <v>44.0095</v>
-      </c>
-      <c r="E8" s="17" t="inlineStr">
-        <is>
-          <t>NIST WebBook.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>CO₂ molar flow during sparge</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>nCO2_rate</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>mol/s</t>
-        </is>
-      </c>
-      <c r="D9" s="49">
-        <f>P_atm*(Q_CO2/1000000/60)/(R_gas*T_K)</f>
-        <v/>
-      </c>
-      <c r="E9" s="14" t="inlineStr">
-        <is>
-          <t>Ideal gas n=PV/RT at surface conditions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>CO₂ per pulse</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>CO2_pulse</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>mol</t>
-        </is>
-      </c>
-      <c r="D10" s="46">
-        <f>nCO2_rate*spg_dur</f>
-        <v/>
-      </c>
-      <c r="E10" s="14" t="inlineStr">
-        <is>
-          <t>Molar flow x duration.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Pulses per hour</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>pulses_h</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>1/h</t>
-        </is>
-      </c>
-      <c r="D11" s="32">
-        <f>60/spg_int</f>
-        <v/>
-      </c>
-      <c r="E11" s="14" t="inlineStr">
-        <is>
-          <t>60 / interval(min).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>Pulses per day</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>pulses_d</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>1/d</t>
-        </is>
-      </c>
-      <c r="D12" s="33">
-        <f>pulses_h*24</f>
-        <v/>
-      </c>
-      <c r="E12" s="14" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="16" t="inlineStr">
-        <is>
-          <t>Average CO₂ supply rate</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>CO2_supply</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>mol/h</t>
-        </is>
-      </c>
-      <c r="D13" s="22">
-        <f>CO2_pulse*pulses_h</f>
-        <v/>
-      </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Time-averaged.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="16" t="inlineStr">
-        <is>
-          <t>CO₂ supply : carbon demand</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>CO2_sd_ratio</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>×</t>
-        </is>
-      </c>
-      <c r="D14" s="32">
-        <f>IF(CO2_cons&gt;0,CO2_supply/CO2_cons,NA())</f>
-        <v/>
-      </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>Carbon supply : demand (~20× = over-dosed, non-limiting). CO₂ mostly bursts at the surface → §11 headspace sweep active from pulse 1. High pCO₂ extends lag (Amer &amp; Kim 2023).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>Sparge duty cycle</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>duty</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D15" s="37">
-        <f>spg_dur/(spg_int*60)</f>
-        <v/>
-      </c>
-      <c r="E15" s="14" t="inlineStr">
-        <is>
-          <t>Fraction of time sparging.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>O₂ accumulated per interval</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>O2_accum</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>mol</t>
-        </is>
-      </c>
-      <c r="D16" s="46">
-        <f>O2_excess/60*spg_int</f>
-        <v/>
-      </c>
-      <c r="E16" s="14" t="inlineStr">
-        <is>
-          <t>Excess O₂ generated between pulses.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>O₂ removable per pulse</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>O2_strip_pulse</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>mol</t>
-        </is>
-      </c>
-      <c r="D17" s="46">
-        <f>strip_sparge/3600*spg_dur</f>
-        <v/>
-      </c>
-      <c r="E17" s="20" t="inlineStr">
-        <is>
-          <t>O₂ a pulse strips (at ceiling).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>Per-pulse balance</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>sched_bal</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>×</t>
-        </is>
-      </c>
-      <c r="D18" s="36">
-        <f>IF(O2_accum&gt;0,O2_strip_pulse/O2_accum,NA())</f>
-        <v/>
-      </c>
-      <c r="E18" s="20" t="inlineStr">
-        <is>
-          <t>&gt;=1 = each pulse clears the interval's O₂ by stripping alone. Bubble path only — the dominant O₂ route is the §11 surface/headspace path; see §14 optimiser.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>Duration floor check</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>dur_ok</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D19" s="45">
-        <f>IF(spg_dur&gt;=pulse_floor,"OK","LOW")</f>
-        <v/>
-      </c>
-      <c r="E19" s="10" t="inlineStr">
-        <is>
-          <t>Pulse must exceed reliable actuation time.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="64" t="inlineStr">
-        <is>
-          <t>IMPORTS (from other tabs)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>(import) EXCESS O₂ to remove</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>O2_excess</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>mol/h</t>
-        </is>
-      </c>
-      <c r="D22" s="61">
-        <f>Biology!$D$9</f>
-        <v/>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>From Biology.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>(import) Temperature (absolute)</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>T_K</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="D23" s="61">
-        <f>Biology!$D$11</f>
-        <v/>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>From Biology.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>(import) Surface pressure</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>P_atm</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Pa</t>
-        </is>
-      </c>
-      <c r="D24" s="61">
-        <f>Biology!$D$12</f>
-        <v/>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>From Biology.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>(import) CO₂ consumed (carbon fixation)</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>CO2_cons</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>mol/h</t>
-        </is>
-      </c>
-      <c r="D25" s="61">
-        <f>Biology!$D$8</f>
-        <v/>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>From Biology.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>(import) Manual sparge interval</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>spg_int_man</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>min</t>
-        </is>
-      </c>
-      <c r="D26" s="60">
-        <f>'Mass Transfer'!$D$60</f>
-        <v/>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>From Mass Transfer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>(import) Schedule mode</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>sched_mode</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D27" s="60">
-        <f>'Mass Transfer'!$D$58</f>
-        <v/>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>From Mass Transfer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>(import) ► OPTIMAL pulse duration</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>spg_dur_opt</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="D28" s="60">
-        <f>'Mass Transfer'!$D$67</f>
-        <v/>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>From Mass Transfer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>(import) O₂ strip rate at ceiling (sparge on)</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>strip_sparge</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>mol/h</t>
-        </is>
-      </c>
-      <c r="D29" s="60">
-        <f>'Mass Transfer'!$D$30</f>
-        <v/>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>From Mass Transfer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>(import) Manual pulse duration</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>spg_dur_man</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="D30" s="60">
-        <f>'Mass Transfer'!$D$59</f>
-        <v/>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>From Mass Transfer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>(import) ► OPTIMAL sparge interval</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>spg_int_opt</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>min</t>
-        </is>
-      </c>
-      <c r="D31" s="60">
-        <f>'Mass Transfer'!$D$68</f>
-        <v/>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>From Mass Transfer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="69" t="inlineStr">
-        <is>
-          <t>REACTOR CALIBRATION (latest date, from CO2 flows)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Reactor (calibration key)</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Reactor</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D34" s="79">
-        <f>Summary!$D$33</f>
-        <v/>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Selects which CO2 flows calibration to use.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>CO2 per pulse (headspace volumes)</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>flush_factor</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Headspace volumes of CO₂ per pulse. 1.0 = exactly one headspace flush (the minimum that fully sweeps it). Raise for margin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>latest calibration date</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>latest_date</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D36" s="80">
-        <f>SUMPRODUCT(MAX(('CO2 flows'!$A$4:$A$200=Reactor)*('CO2 flows'!$J$4:$J$200&gt;0)*'CO2 flows'!$B$4:$B$200))</f>
-        <v/>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Latest date for this reactor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>flowrate (calibrated)</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>flowrate_cal</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>ml/s</t>
-        </is>
-      </c>
-      <c r="D37" s="80">
-        <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$200=Reactor)*('CO2 flows'!$B$4:$B$200=latest_date)*'CO2 flows'!$J$4:$J$200)/MAX(1,SUMPRODUCT(('CO2 flows'!$A$4:$A$200=Reactor)*('CO2 flows'!$B$4:$B$200=latest_date)*('CO2 flows'!$J$4:$J$200&gt;0)*1))</f>
-        <v/>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Pulled from CO2 flows (latest date for reactor).</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>min sparge (calibrated)</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>min_sparge_cal</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="D38" s="80">
-        <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$200=Reactor)*('CO2 flows'!$B$4:$B$200=latest_date)*'CO2 flows'!$I$4:$I$200)/MAX(1,SUMPRODUCT(('CO2 flows'!$A$4:$A$200=Reactor)*('CO2 flows'!$B$4:$B$200=latest_date)*('CO2 flows'!$J$4:$J$200&gt;0)*1))</f>
-        <v/>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Pulled from CO2 flows (latest date for reactor).</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>reactor has a calibration row?</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>has_cal</t>
-        </is>
-      </c>
-      <c r="D39" s="80">
-        <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$200=Reactor)*('CO2 flows'!$J$4:$J$200&gt;0)*1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="D40" s="80" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>calibration source</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>cal_warning</t>
-        </is>
-      </c>
-      <c r="D41" s="80">
-        <f>IF(has_cal&gt;0,"calibrated: "&amp;Reactor,"NO CALIBRATION for "&amp;Reactor&amp;" - add a row in CO2 flows with nominal flowrate + minimum sparge")</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="D14">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="num" val="1"/>
-        <cfvo type="num" val="5"/>
-        <cfvo type="num" val="20"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D19">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
-      <formula>"LOW"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="4" dxfId="11">
-      <formula>OR(ISNUMBER(SEARCH("RISK",D19)),ISNUMBER(SEARCH("OVER",D19)),ISNUMBER(SEARCH("BELOW",D19)),ISNUMBER(SEARCH("EXCEED",D19)),ISNUMBER(SEARCH("NO CALIB",D19)),ISNUMBER(SEARCH("NEAREST",D19)),ISNUMBER(SEARCH("EXPLOSIVE",D19)),ISNUMBER(SEARCH("LOW",D19)),ISNUMBER(SEARCH("TIGHT",D19)),ISNUMBER(SEARCH("insufficient",D19)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="5" dxfId="12">
-      <formula>OR(ISNUMBER(SEARCH("OK",D19)),ISNUMBER(SEARCH("calibrated",D19)),ISNUMBER(SEARCH("under optimum",D19)),ISNUMBER(SEARCH("above min",D19)),ISNUMBER(SEARCH("exact",D19)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D41">
-    <cfRule type="expression" priority="6" dxfId="11">
-      <formula>OR(ISNUMBER(SEARCH("RISK",D41)),ISNUMBER(SEARCH("OVER",D41)),ISNUMBER(SEARCH("BELOW",D41)),ISNUMBER(SEARCH("EXCEED",D41)),ISNUMBER(SEARCH("NO CALIB",D41)),ISNUMBER(SEARCH("NEAREST",D41)),ISNUMBER(SEARCH("EXPLOSIVE",D41)),ISNUMBER(SEARCH("LOW",D41)),ISNUMBER(SEARCH("TIGHT",D41)),ISNUMBER(SEARCH("insufficient",D41)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="7" dxfId="12">
-      <formula>OR(ISNUMBER(SEARCH("OK",D41)),ISNUMBER(SEARCH("calibrated",D41)),ISNUMBER(SEARCH("under optimum",D41)),ISNUMBER(SEARCH("above min",D41)),ISNUMBER(SEARCH("exact",D41)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation sqref="D58" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
-      <formula1>"Manual,Optimal"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor theme="9"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:Q75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
model(modular): selectors to top of Summary (reactor name/electrode/organism/media), porosity demoted, CF reapplied
- D3-D6 are now the experiment dropdowns: Reactor (ed04 by name), Electrode, HOB organism, Media; wiring repointed to them
- sinter porosity grade demoted to a scalar input (only relevant when sparger=Sintered); sparger/version no longer shown as top inputs
- traffic-light conditional formatting reapplied to all Summary output flags (D7:D20, D44:D51, D63:D65)
- removed stale Summary rx_ver/sparger names; verified: no #REF, all names resolve, dropdowns valid, headline numbers unchanged

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel-modular.xlsx
+++ b/Media/electroPioreactorGasModel-modular.xlsx
@@ -14,14 +14,16 @@
     <sheet name="CO2 flows" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="por_grade" localSheetId="0">Summary!$D$5</definedName>
-    <definedName name="rx_ver" localSheetId="0">Summary!$D$3</definedName>
-    <definedName name="sparger" localSheetId="0">Summary!$D$4</definedName>
     <definedName name="led_intensity" localSheetId="0">Summary!$D$37</definedName>
     <definedName name="stir_rpm_set" localSheetId="0">Summary!$D$38</definedName>
     <definedName name="media_volume" localSheetId="0">Summary!$D$39</definedName>
     <definedName name="temp_C" localSheetId="0">Summary!$D$40</definedName>
     <definedName name="P_atm_set" localSheetId="0">Summary!$D$41</definedName>
+    <definedName name="Reactor_sel" localSheetId="0">Summary!$D$3</definedName>
+    <definedName name="electrode_sel" localSheetId="0">Summary!$D$4</definedName>
+    <definedName name="organism_sel" localSheetId="0">Summary!$D$5</definedName>
+    <definedName name="media_sel" localSheetId="0">Summary!$D$6</definedName>
+    <definedName name="por_grade" localSheetId="0">Summary!$D$42</definedName>
     <definedName name="A_x" localSheetId="1">Geometry!$D$21</definedName>
     <definedName name="D_int" localSheetId="1">Geometry!$D$22</definedName>
     <definedName name="D_int_1" localSheetId="1">Geometry!$D$12</definedName>
@@ -712,7 +714,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -845,6 +847,9 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1209,7 +1214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T65"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1255,12 +1260,12 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>Reactor version (resolved from reactor)</t>
+          <t>Reactor (select)</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>rx_ver</t>
+          <t>Reactor_sel</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
@@ -1268,9 +1273,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D3" s="75">
-        <f>Geometry!$D$51</f>
-        <v/>
+      <c r="D3" s="98" t="inlineStr">
+        <is>
+          <t>ed04</t>
+        </is>
       </c>
       <c r="E3" s="10" t="inlineStr">
         <is>
@@ -1281,12 +1287,12 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Sparger type (resolved from electrode)</t>
+          <t>Electrode (select)</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>sparger</t>
+          <t>electrode_sel</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
@@ -1294,9 +1300,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D4" s="82">
-        <f>Electrochemistry!$D$31</f>
-        <v/>
+      <c r="D4" s="99" t="inlineStr">
+        <is>
+          <t>MMO tube</t>
+        </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
@@ -1307,12 +1314,12 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Sinter porosity grade (if Sintered)</t>
+          <t>HOB organism (select)</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>por_grade</t>
+          <t>organism_sel</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -1320,8 +1327,10 @@
           <t>0-5</t>
         </is>
       </c>
-      <c r="D5" s="30" t="n">
-        <v>5</v>
+      <c r="D5" s="100" t="inlineStr">
+        <is>
+          <t>Cupriavidus necator</t>
+        </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
@@ -1329,7 +1338,23 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Media (select)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>media_sel</t>
+        </is>
+      </c>
+      <c r="D6" s="88" t="inlineStr">
+        <is>
+          <t>Sydow 2017 minimal</t>
+        </is>
+      </c>
+    </row>
     <row r="7">
       <c r="A7" s="59" t="inlineStr">
         <is>
@@ -1623,7 +1648,6 @@
       <c r="C30" s="28" t="n"/>
       <c r="D30" s="29" t="n"/>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="73" t="inlineStr">
         <is>
@@ -1631,74 +1655,6 @@
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Reactor</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Reactor_sel</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>ed04</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Electrode</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>electrode_sel</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>MMO tube</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>HOB organism</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>organism_sel</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Cupriavidus necator</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>media_sel</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Sydow 2017 minimal</t>
-        </is>
-      </c>
-    </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
@@ -1792,7 +1748,21 @@
         <v>101325</v>
       </c>
     </row>
-    <row r="42"/>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Sinter porosity grade (only if sparger = Sintered)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>por_grade</t>
+        </is>
+      </c>
+      <c r="D42" s="88" t="n">
+        <v>5</v>
+      </c>
+    </row>
     <row r="43">
       <c r="A43" s="69" t="inlineStr">
         <is>
@@ -1917,7 +1887,6 @@
         <v/>
       </c>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="69" t="inlineStr">
         <is>
@@ -2094,7 +2063,6 @@
         </is>
       </c>
     </row>
-    <row r="61"/>
     <row r="62">
       <c r="A62" s="69" t="inlineStr">
         <is>
@@ -2151,6 +2119,12 @@
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="12">
       <formula>OR(ISNUMBER(SEARCH("OK",D7)),ISNUMBER(SEARCH("calibrated",D7)),ISNUMBER(SEARCH("under optimum",D7)),ISNUMBER(SEARCH("above min",D7)),ISNUMBER(SEARCH("exact",D7)))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="11" stopIfTrue="0">
+      <formula>OR(ISNUMBER(SEARCH("RISK",D7)),ISNUMBER(SEARCH("OVER",D7)),ISNUMBER(SEARCH("BELOW",D7)),ISNUMBER(SEARCH("EXCEED",D7)),ISNUMBER(SEARCH("NO CALIB",D7)),ISNUMBER(SEARCH("NEAREST",D7)),ISNUMBER(SEARCH("EXPLOSIVE",D7)),ISNUMBER(SEARCH("TIGHT",D7)),ISNUMBER(SEARCH("insufficient",D7)),EXACT(D7,"LOW"))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="12" stopIfTrue="0">
+      <formula>OR(EXACT(D7,"OK"),ISNUMBER(SEARCH("calibrated",D7)),ISNUMBER(SEARCH("under optimum",D7)),ISNUMBER(SEARCH("above min",D7)),ISNUMBER(SEARCH("exact",D7)),ISNUMBER(SEARCH("CARBON-limited",D7)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D44:D51">
@@ -2160,22 +2134,36 @@
     <cfRule type="expression" priority="4" dxfId="12">
       <formula>OR(ISNUMBER(SEARCH("OK",D44)),ISNUMBER(SEARCH("calibrated",D44)),ISNUMBER(SEARCH("under optimum",D44)),ISNUMBER(SEARCH("above min",D44)),ISNUMBER(SEARCH("exact",D44)))</formula>
     </cfRule>
+    <cfRule type="expression" priority="7" dxfId="11" stopIfTrue="0">
+      <formula>OR(ISNUMBER(SEARCH("RISK",D44)),ISNUMBER(SEARCH("OVER",D44)),ISNUMBER(SEARCH("BELOW",D44)),ISNUMBER(SEARCH("EXCEED",D44)),ISNUMBER(SEARCH("NO CALIB",D44)),ISNUMBER(SEARCH("NEAREST",D44)),ISNUMBER(SEARCH("EXPLOSIVE",D44)),ISNUMBER(SEARCH("TIGHT",D44)),ISNUMBER(SEARCH("insufficient",D44)),EXACT(D44,"LOW"))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="12" stopIfTrue="0">
+      <formula>OR(EXACT(D44,"OK"),ISNUMBER(SEARCH("calibrated",D44)),ISNUMBER(SEARCH("under optimum",D44)),ISNUMBER(SEARCH("above min",D44)),ISNUMBER(SEARCH("exact",D44)),ISNUMBER(SEARCH("CARBON-limited",D44)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D63:D65">
+    <cfRule type="expression" priority="9" dxfId="11" stopIfTrue="0">
+      <formula>OR(ISNUMBER(SEARCH("RISK",D63)),ISNUMBER(SEARCH("OVER",D63)),ISNUMBER(SEARCH("BELOW",D63)),ISNUMBER(SEARCH("EXCEED",D63)),ISNUMBER(SEARCH("NO CALIB",D63)),ISNUMBER(SEARCH("NEAREST",D63)),ISNUMBER(SEARCH("EXPLOSIVE",D63)),ISNUMBER(SEARCH("TIGHT",D63)),ISNUMBER(SEARCH("insufficient",D63)),EXACT(D63,"LOW"))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="12" stopIfTrue="0">
+      <formula>OR(EXACT(D63,"OK"),ISNUMBER(SEARCH("calibrated",D63)),ISNUMBER(SEARCH("under optimum",D63)),ISNUMBER(SEARCH("above min",D63)),ISNUMBER(SEARCH("exact",D63)),ISNUMBER(SEARCH("CARBON-limited",D63)))</formula>
+    </cfRule>
   </conditionalFormatting>
   <dataValidations count="5">
-    <dataValidation sqref="D5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
-      <formula1>"0,1,2,3,4,5"</formula1>
-    </dataValidation>
-    <dataValidation sqref="D33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Geometry!$A$59:$A$88</formula1>
     </dataValidation>
-    <dataValidation sqref="D34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Electrochemistry!$A$35:$A$43</formula1>
     </dataValidation>
-    <dataValidation sqref="D35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Biology!$A$52:$A$65</formula1>
     </dataValidation>
-    <dataValidation sqref="D36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Biology!$A$61:$A$69</formula1>
+    </dataValidation>
+    <dataValidation sqref="D42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"0,1,2,3,4,5"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2190,7 +2178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T87"/>
+  <dimension ref="A1:I87"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2267,7 +2255,7 @@
         </is>
       </c>
       <c r="D5" s="79">
-        <f>Summary!$D$33</f>
+        <f>Summary!$D$3</f>
         <v/>
       </c>
       <c r="E5" t="inlineStr">
@@ -3472,7 +3460,6 @@
         <v/>
       </c>
     </row>
-    <row r="56"/>
     <row r="57">
       <c r="A57" s="73" t="inlineStr">
         <is>
@@ -3756,7 +3743,6 @@
         </is>
       </c>
     </row>
-    <row r="81"/>
     <row r="82">
       <c r="A82" s="73" t="inlineStr">
         <is>
@@ -3963,7 +3949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T39"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4113,7 +4099,7 @@
         </is>
       </c>
       <c r="D8" s="79">
-        <f>Summary!$D$34</f>
+        <f>Summary!$D$4</f>
         <v/>
       </c>
     </row>
@@ -4864,7 +4850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T61"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5014,7 +5000,7 @@
         </is>
       </c>
       <c r="D8" s="79">
-        <f>Summary!$D$35</f>
+        <f>Summary!$D$5</f>
         <v/>
       </c>
     </row>
@@ -6307,7 +6293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T132"/>
+  <dimension ref="A1:E132"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6775,7 +6761,7 @@
         </is>
       </c>
       <c r="D20" s="94">
-        <f>Summary!$D$5</f>
+        <f>Summary!$D$42</f>
         <v/>
       </c>
       <c r="E20" t="inlineStr">
@@ -9440,7 +9426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T75"/>
+  <dimension ref="A1:Q75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="9"/>
@@ -10739,7 +10725,6 @@
     <row r="47">
       <c r="B47" s="66" t="n"/>
     </row>
-    <row r="48"/>
     <row r="49">
       <c r="A49" s="73" t="n"/>
     </row>
@@ -10756,34 +10741,15 @@
     <row r="52">
       <c r="A52" s="72" t="n"/>
     </row>
-    <row r="53"/>
     <row r="54">
       <c r="A54" s="73" t="n"/>
     </row>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="72" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="72" t="n"/>
     </row>
-    <row r="74"/>
     <row r="75">
       <c r="A75" s="73" t="n"/>
     </row>

</xml_diff>

<commit_message>
model(modular): fix Reactor calibration key left pointing at cleared D33 -> D3
Moving the reactor selector to D3 repointed Geometry's reactor_sel but missed the
calibration Reactor cell (folded from Dosing into Mass Transfer), which still read the
now-empty old D33 -> Reactor='0' -> no calibration -> flowrate_cal 0 -> #DIV/0! across
the schedule. Repointed MT Reactor to Summary D3; confirmed no other stale D33-36 refs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel-modular.xlsx
+++ b/Media/electroPioreactorGasModel-modular.xlsx
@@ -1648,6 +1648,7 @@
       <c r="C30" s="28" t="n"/>
       <c r="D30" s="29" t="n"/>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="73" t="inlineStr">
         <is>
@@ -1655,6 +1656,10 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
@@ -1887,6 +1892,7 @@
         <v/>
       </c>
     </row>
+    <row r="52"/>
     <row r="53">
       <c r="A53" s="69" t="inlineStr">
         <is>
@@ -2063,6 +2069,7 @@
         </is>
       </c>
     </row>
+    <row r="61"/>
     <row r="62">
       <c r="A62" s="69" t="inlineStr">
         <is>
@@ -3460,6 +3467,7 @@
         <v/>
       </c>
     </row>
+    <row r="56"/>
     <row r="57">
       <c r="A57" s="73" t="inlineStr">
         <is>
@@ -3743,6 +3751,7 @@
         </is>
       </c>
     </row>
+    <row r="81"/>
     <row r="82">
       <c r="A82" s="73" t="inlineStr">
         <is>
@@ -9057,7 +9066,7 @@
         </is>
       </c>
       <c r="D115" s="79">
-        <f>Summary!$D$33</f>
+        <f>Summary!$D$3</f>
         <v/>
       </c>
     </row>
@@ -10725,6 +10734,7 @@
     <row r="47">
       <c r="B47" s="66" t="n"/>
     </row>
+    <row r="48"/>
     <row r="49">
       <c r="A49" s="73" t="n"/>
     </row>
@@ -10741,15 +10751,34 @@
     <row r="52">
       <c r="A52" s="72" t="n"/>
     </row>
+    <row r="53"/>
     <row r="54">
       <c r="A54" s="73" t="n"/>
     </row>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
     <row r="72">
       <c r="A72" s="72" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="72" t="n"/>
     </row>
+    <row r="74"/>
     <row r="75">
       <c r="A75" s="73" t="n"/>
     </row>

</xml_diff>

<commit_message>
model(modular): O2 Henry constant -> 1.2e-5 (Sander 2023); provisional-pulse note; remove old single-sheet file
- Biology H_O2ref 1.3e-5 -> 1.2e-5 (Sander 2023), cited in col E; reproduces ~7.5 mg/L air-saturation at 30C, O2 inhibition ceiling 11.6 -> 10.7 mg/L, O2-limited interval 1.39 -> 1.29 min
- Summary note: headspace & optimal pulse PROVISIONAL pending a fill-to-septum vial measurement (B1; geometry-consistency cell flags INCONSISTENT until reconciled)
- deleted the superseded single-sheet Media/electroPioreactorGasModel.xlsx so no one opens the wrong file (git history retains it)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel-modular.xlsx
+++ b/Media/electroPioreactorGasModel-modular.xlsx
@@ -715,7 +715,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -858,6 +858,7 @@
     <xf numFmtId="0" fontId="21" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1598,9 +1599,9 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Literature-supported (~90%)</t>
+      <c r="A23" s="104" t="inlineStr">
+        <is>
+          <t>NOTE: headspace &amp; optimal pulse are PROVISIONAL pending a fill-to-septum vial measurement (see Geometry consistency check)</t>
         </is>
       </c>
     </row>
@@ -5343,11 +5344,11 @@
         </is>
       </c>
       <c r="D21" s="44" t="n">
-        <v>1.3e-05</v>
+        <v>1.2e-05</v>
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>Sander (2023) compilation (supersedes 2015), value from Burkholder et al. 2019.</t>
+          <t>Sander (2023) recommended H^cp O2; reproduces ~7.5 mg/L air-saturation at 30 degC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(protocols): add experiment-protocol set + index, hyperlinked from the model
Eight standalone bench SOPs in Media/protocols/, each with an optimal and a budget route and tied to the exact model cell it feeds:
- vial-geometry (B1 headspace blocker), surface-kla (#1 sensitivity), faradaic-efficiency (etaF), dissolved-oxygen (organism DO bands), flow-calibration (per-reactor CO2), knallgas-stoichiometry (H2:O2:CO2 uptake), sinter-porosity (por_grade), gerrit-current (LED->current)
- README.md index: leverage-ordered table mapping each protocol to its model cell, current state, and why; plus an ambient-pressure note and how-to
- Summary: protocol hyperlinks on the ranked-improvements rows + the geometry-check row, and a master index link
All methods web-grounded with cited sources; spreadsheet verified (independent gate passes, headline numbers unchanged).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel-modular.xlsx
+++ b/Media/electroPioreactorGasModel-modular.xlsx
@@ -284,7 +284,7 @@
     <numFmt numFmtId="171" formatCode="0.0000000"/>
     <numFmt numFmtId="172" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="28">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -436,6 +436,11 @@
     </font>
     <font>
       <color rgb="FF7030A0"/>
+    </font>
+    <font>
+      <color rgb="FF0000FF"/>
+      <sz val="9"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="17">
@@ -716,7 +721,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="111">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -876,6 +881,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1607,6 +1613,10 @@
         <f>Geometry!$D$90</f>
         <v/>
       </c>
+      <c r="E21" s="111">
+        <f>HYPERLINK("protocols/vial-geometry.md","→ vial-geometry.md")</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="101" t="inlineStr">
@@ -1937,6 +1947,10 @@
           <t>Effort</t>
         </is>
       </c>
+      <c r="D53" s="111">
+        <f>HYPERLINK("protocols/README.md","all protocols →")</f>
+        <v/>
+      </c>
       <c r="E53" s="69" t="inlineStr">
         <is>
           <t>Why it matters</t>
@@ -1959,6 +1973,10 @@
           <t>med</t>
         </is>
       </c>
+      <c r="D54" s="111">
+        <f>HYPERLINK("protocols/surface-kla.md","protocol →")</f>
+        <v/>
+      </c>
       <c r="E54" t="inlineStr">
         <is>
           <t>375% sensitivity; decides whether DO stays in the organism band</t>
@@ -1981,6 +1999,10 @@
           <t>med</t>
         </is>
       </c>
+      <c r="D55" s="111">
+        <f>HYPERLINK("protocols/faradaic-efficiency.md","protocol →")</f>
+        <v/>
+      </c>
       <c r="E55" t="inlineStr">
         <is>
           <t>sets the H2/O2 split and net O2; currently assumed 1.0</t>
@@ -2003,6 +2025,10 @@
           <t>low</t>
         </is>
       </c>
+      <c r="D56" s="111">
+        <f>HYPERLINK("protocols/dissolved-oxygen.md","protocol →")</f>
+        <v/>
+      </c>
       <c r="E56" t="inlineStr">
         <is>
           <t>lower DO guardrail; currently a gap for every organism</t>
@@ -2025,6 +2051,10 @@
           <t>low</t>
         </is>
       </c>
+      <c r="D57" s="111">
+        <f>HYPERLINK("protocols/flow-calibration.md","protocol →")</f>
+        <v/>
+      </c>
       <c r="E57" t="inlineStr">
         <is>
           <t>each experiment; only ed04 calibrated so far</t>
@@ -2047,6 +2077,10 @@
           <t>high</t>
         </is>
       </c>
+      <c r="D58" s="111">
+        <f>HYPERLINK("protocols/knallgas-stoichiometry.md","protocol →")</f>
+        <v/>
+      </c>
       <c r="E58" t="inlineStr">
         <is>
           <t>carbon/O2 balance; needs a growing culture</t>
@@ -2069,6 +2103,10 @@
           <t>low</t>
         </is>
       </c>
+      <c r="D59" s="111">
+        <f>HYPERLINK("protocols/sinter-porosity.md","protocol →")</f>
+        <v/>
+      </c>
       <c r="E59" t="inlineStr">
         <is>
           <t>bubble size when sparger = sintered</t>
@@ -2090,6 +2128,10 @@
         <is>
           <t>low</t>
         </is>
+      </c>
+      <c r="D60" s="111">
+        <f>HYPERLINK("protocols/README.md","protocol →")</f>
+        <v/>
       </c>
       <c r="E60" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
model(modular): electrode = single 'MMO Tubular' (porosity 0), per Gerrit's actual sourced disc
Replaced the speculative MMO tube 0-5 with the one electrode we actually have: MMO Tubular, Sintered, sinter-porosity grade 0 - from Gerrit's order of 8mm porosity-0 sintered discs (SD8/0/P; stock fallback SD10/0/P; Scientific Glass Labs, 2026-05), cited in col E. VLOOKUP ranges back to A35:A37; default electrode + dropdown updated. Grade 0 is the coarsest, so the 'Sinter OOR' bubble flag is expected (honest).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel-modular.xlsx
+++ b/Media/electroPioreactorGasModel-modular.xlsx
@@ -283,7 +283,7 @@
     <numFmt numFmtId="170" formatCode="0.0000000"/>
     <numFmt numFmtId="171" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="29">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -455,6 +455,10 @@
     <font>
       <b val="1"/>
       <color rgb="FF0000FF"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="17">
@@ -732,7 +736,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -890,6 +894,7 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="171" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1401,7 +1406,7 @@
       </c>
       <c r="D4" s="104" t="inlineStr">
         <is>
-          <t>MMO tube 5</t>
+          <t>MMO Tubular</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
@@ -2287,7 +2292,7 @@
       <formula1>=Geometry!$A$59:$A$80</formula1>
     </dataValidation>
     <dataValidation sqref="D4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Electrochemistry!$A$35:$A$42</formula1>
+      <formula1>=Electrochemistry!$A$35:$A$37</formula1>
     </dataValidation>
     <dataValidation sqref="D5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Biology!$A$52:$A$57</formula1>
@@ -4706,7 +4711,7 @@
         </is>
       </c>
       <c r="D27" s="69">
-        <f>VLOOKUP(electrode_sel,$A$35:$I$42,9,FALSE)</f>
+        <f>VLOOKUP(electrode_sel,$A$35:$I$37,9,FALSE)</f>
         <v/>
       </c>
       <c r="E27" s="23" t="inlineStr">
@@ -4786,7 +4791,7 @@
         </is>
       </c>
       <c r="D31" s="72">
-        <f>VLOOKUP(electrode_sel,$A$35:$I$42,4,FALSE)</f>
+        <f>VLOOKUP(electrode_sel,$A$35:$I$37,4,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -4802,8 +4807,13 @@
         </is>
       </c>
       <c r="D32" s="105">
-        <f>IF(ISNUMBER(VLOOKUP(electrode_sel,$A$35:$I$42,5,FALSE)),VLOOKUP(electrode_sel,$A$35:$I$42,5,FALSE),0)</f>
-        <v/>
+        <f>IF(ISNUMBER(VLOOKUP(electrode_sel,$A$35:$I$37,5,FALSE)),VLOOKUP(electrode_sel,$A$35:$I$37,5,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="E32" s="109" t="inlineStr">
+        <is>
+          <t>Porosity 0 = Gerrit's sourced sintered disc (SD8/0/P 8mm, fallback SD10/0/P 10mm; Scientific Glass Labs, 2026-05)</t>
+        </is>
       </c>
       <c r="H32" s="68" t="n"/>
     </row>
@@ -4946,7 +4956,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>MMO tube 0</t>
+          <t>MMO Tubular</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4983,200 +4993,14 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>MMO tube 1</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>MMO</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>6</v>
-      </c>
-      <c r="D38" s="71" t="inlineStr">
-        <is>
-          <t>Sintered</t>
-        </is>
-      </c>
-      <c r="E38" t="n">
-        <v>1</v>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>SS rod</t>
-        </is>
-      </c>
-      <c r="G38" t="n">
-        <v>6</v>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="I38" t="n">
-        <v>2</v>
-      </c>
+      <c r="D38" s="71" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>MMO tube 2</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>MMO</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>6</v>
-      </c>
-      <c r="D39" s="72" t="inlineStr">
-        <is>
-          <t>Sintered</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>2</v>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>SS rod</t>
-        </is>
-      </c>
-      <c r="G39" t="n">
-        <v>6</v>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="I39" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>MMO tube 3</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>MMO</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>6</v>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Sintered</t>
-        </is>
-      </c>
-      <c r="E40" t="n">
-        <v>3</v>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>SS rod</t>
-        </is>
-      </c>
-      <c r="G40" t="n">
-        <v>6</v>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="I40" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>MMO tube 4</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>MMO</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>6</v>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Sintered</t>
-        </is>
-      </c>
-      <c r="E41" t="n">
-        <v>4</v>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>SS rod</t>
-        </is>
-      </c>
-      <c r="G41" t="n">
-        <v>6</v>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="I41" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>MMO tube 5</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>MMO</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>6</v>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Sintered</t>
-        </is>
-      </c>
-      <c r="E42" t="n">
-        <v>5</v>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>SS rod</t>
-        </is>
-      </c>
-      <c r="G42" t="n">
-        <v>6</v>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="I42" t="n">
-        <v>2</v>
-      </c>
-    </row>
+      <c r="D39" s="72" t="n"/>
+    </row>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
   </sheetData>
   <conditionalFormatting sqref="D13">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">

</xml_diff>

<commit_message>
model(modular): sparge interval credits surface O2 stripping (kL_surf proxy), not zero
duty_O2vent and spg_int_max now use MAX(0, O2_net_gen - surf_strip) instead of O2_net_gen - i.e. the sparge only has to vent the O2 that surface stripping (from the kL_surf proxy) does not. When surface handles the O2 the interval becomes carbon-limited; below ~150 rpm it goes O2-limited and shortens sharply, so the stirrer now affects the headline interval. Refine via the kL_surf measurement. Earlier behaviour (assuming surface stripping = 0) over-sparged ~125x.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel-modular.xlsx
+++ b/Media/electroPioreactorGasModel-modular.xlsx
@@ -1986,7 +1986,7 @@
       </c>
       <c r="F15" s="21" t="inlineStr">
         <is>
-          <t>Time between doses (conservative, O2-safe). The 'interval can be relaxed?' check below says if you can dose less often.</t>
+          <t>Time between doses. Now credits surface O2 stripping (kL_surf proxy); when surface handles the O2 this is carbon-limited. Refine via the kL_surf measurement.</t>
         </is>
       </c>
     </row>
@@ -10131,12 +10131,12 @@
         </is>
       </c>
       <c r="D87" s="61">
-        <f>O2_net_gen/(target_DO_frac*(O2_ceil_Pa/P_atm))/(nCO2_rate*3600)</f>
+        <f>MAX(0,O2_net_gen-surf_strip)/(target_DO_frac*(O2_ceil_Pa/P_atm))/(nCO2_rate*3600)</f>
         <v/>
       </c>
       <c r="E87" s="131" t="inlineStr">
         <is>
-          <t>Duty so the vented CO₂ throughput carries the worst-case (lag, no uptake) net O₂ out at ≤ target DO. Usually the binding floor.</t>
+          <t>O2 the sparge must vent = net O2 minus surface stripping (proxy); 0 when surface stripping alone holds DO</t>
         </is>
       </c>
       <c r="F87" s="20" t="n"/>
@@ -10185,12 +10185,12 @@
         </is>
       </c>
       <c r="D89" s="61">
-        <f>target_DO_frac*t_O2_ceiling_lag</f>
+        <f>target_DO_frac*O2_ceil_C*(V_charge/1000000)/MAX(0.000000000001,O2_net_gen-surf_strip)*60</f>
         <v/>
       </c>
       <c r="E89" s="131" t="inlineStr">
         <is>
-          <t>Pulses must be frequent enough that DO doesn't spike past target between flushes (lag worst-case).</t>
+          <t>O2-limited interval, now crediting surface stripping (surf_strip from the kL_surf proxy) rather than assuming zero; refine by measuring kL_surf</t>
         </is>
       </c>
       <c r="F89" s="20" t="n"/>

</xml_diff>

<commit_message>
model(modular): fix CF red token 'UNDER' reddening 'at/under optimum' and 'holds DO under'
Renamed D26's shortfall state to 'SHORTFALL (CO2 < demand)' and replaced the generic 'UNDER' red token with 'SHORTFALL'; D21/D23 now go green.
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel-modular.xlsx
+++ b/Media/electroPioreactorGasModel-modular.xlsx
@@ -1142,7 +1142,7 @@
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
     <cellStyle name="Neutral" xfId="3" builtinId="28"/>
   </cellStyles>
-  <dxfs count="23">
+  <dxfs count="26">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1318,6 +1318,30 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+          <bgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFEB9C"/>
+          <bgColor rgb="00FFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+          <bgColor rgb="00C6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2204,7 +2228,7 @@
       <c r="B26" s="20" t="n"/>
       <c r="C26" s="20" t="n"/>
       <c r="D26" s="118">
-        <f>IFERROR(IF('Mass Transfer'!$D$126&gt;=1,"OK","UNDER (CO2 &lt; demand)"),"calibrate this reactor first")</f>
+        <f>IFERROR(IF('Mass Transfer'!$D$126&gt;=1,"OK","SHORTFALL (CO2 &lt; demand)"),"calibrate this reactor first")</f>
         <v/>
       </c>
       <c r="E26" s="24">
@@ -2951,14 +2975,14 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D19:D33">
-    <cfRule type="expression" priority="11" dxfId="15" stopIfTrue="1">
-      <formula>OR(ISNUMBER(SEARCH("INCONSISTENT",D19)),ISNUMBER(SEARCH("OVER",D19)),ISNUMBER(SEARCH("BELOW",D19)),ISNUMBER(SEARCH("EXCEED",D19)),ISNUMBER(SEARCH("NO CALIB",D19)),ISNUMBER(SEARCH("calibrate this",D19)),ISNUMBER(SEARCH("RISK",D19)),ISNUMBER(SEARCH("EXPLOSIVE",D19)),ISNUMBER(SEARCH("OOR",D19)),ISNUMBER(SEARCH("insufficient",D19)),ISNUMBER(SEARCH("TIP SPEED",D19)),ISNUMBER(SEARCH("UNDER",D19)),EXACT(D19,"OUT"),EXACT(D19,"LOW"))</formula>
+    <cfRule type="expression" priority="11" dxfId="23" stopIfTrue="1">
+      <formula>OR(ISNUMBER(SEARCH("INCONSISTENT",D19)),ISNUMBER(SEARCH("OVER",D19)),ISNUMBER(SEARCH("BELOW",D19)),ISNUMBER(SEARCH("EXCEED",D19)),ISNUMBER(SEARCH("NO CALIB",D19)),ISNUMBER(SEARCH("calibrate this",D19)),ISNUMBER(SEARCH("RISK",D19)),ISNUMBER(SEARCH("EXPLOSIVE",D19)),ISNUMBER(SEARCH("OOR",D19)),ISNUMBER(SEARCH("insufficient",D19)),ISNUMBER(SEARCH("TIP SPEED",D19)),ISNUMBER(SEARCH("SHORTFALL",D19)),EXACT(D19,"OUT"),EXACT(D19,"LOW"))</formula>
     </cfRule>
-    <cfRule type="expression" priority="12" dxfId="14" stopIfTrue="1">
+    <cfRule type="expression" priority="12" dxfId="24" stopIfTrue="1">
       <formula>OR(ISNUMBER(SEARCH("above optimum",D19)),ISNUMBER(SEARCH("watch",D19)),ISNUMBER(SEARCH("NEAREST",D19)),ISNUMBER(SEARCH("unknown",D19)),ISNUMBER(SEARCH("TIGHT",D19)))</formula>
     </cfRule>
-    <cfRule type="expression" priority="13" dxfId="13" stopIfTrue="1">
-      <formula>OR(EXACT(D19,"OK"),ISNUMBER(SEARCH("calibrated:",D19)),ISNUMBER(SEARCH("under optimum",D19)),ISNUMBER(SEARCH("above min",D19)),ISNUMBER(SEARCH("CARBON-limited",D19)),ISNUMBER(SEARCH("Static",D19)),ISNUMBER(SEARCH("Dynamic",D19)))</formula>
+    <cfRule type="expression" priority="13" dxfId="25" stopIfTrue="1">
+      <formula>OR(EXACT(D19,"OK"),ISNUMBER(SEARCH("calibrated:",D19)),ISNUMBER(SEARCH("optimum",D19)),ISNUMBER(SEARCH("above min",D19)),ISNUMBER(SEARCH("CARBON-limited",D19)),ISNUMBER(SEARCH("Static",D19)),ISNUMBER(SEARCH("Dynamic",D19)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">

</xml_diff>